<commit_message>
Quadro Free: regola personalizzabile e consigli sui pocket
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quadro/Quadro-Free.xlsx
+++ b/quadro/Quadro-Free.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +147,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -890,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -910,7 +913,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Your money, in four. Give every euro a job: 55% Essentials · 20% Quality of Life · 15% Safety Fund · 10% Investments.</t>
+          <t>Your money, in four. Give every euro a job. My suggested split: 55% Essentials · 20% Quality of Life · 15% Safety Fund · 10% Investments. Your rule, your call.</t>
         </is>
       </c>
     </row>
@@ -940,7 +943,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Set the year, the day your month starts (e.g. your payday) and your categories. Want a different rule? Change the percentages: they just need to add up to 100%.</t>
+          <t>Set the year, the day your month starts (e.g. your payday) and your categories. Then choose your rule: 55-20-15-10 is what I recommend, but you decide (e.g. 50-30-10-10 or 60-15-15-10). The percentages just need to add up to 100%.</t>
         </is>
       </c>
     </row>
@@ -994,27 +997,78 @@
     </row>
     <row r="12"/>
     <row r="13">
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Make it real: one pocket per bucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>The plan works best when the money is really split. On payday, move each bucket's share to its own place, so what's in it is what you can spend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Revolut</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Easiest way: create 4 Pockets (Essentials, Quality of Life, Safety Fund, Investments) and set a scheduled transfer on payday for each share. Pay bills from the Essentials pocket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Trade Republic</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Great for the Investments bucket: set a savings plan (PAC) on ETFs for your 10% and track it in the Investments sheet. Cash waiting to be invested earns interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Other banks</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Use sub-accounts or “spaces” if your bank has them (e.g. N26 Spaces, bunq, Monzo Pots). If not, open a second free account for savings and keep Essentials + Quality of Life in the main one: set a standing order on payday for the Safety Fund and Investments shares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Tip: type only in the yellow cells; grey cells calculate themselves. Calculations are protected so they can't be broken by accident.</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="20"/>
+    <row r="21" ht="32" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Go Pro</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>All 12 months · leftovers that roll over · recurring payments · other currencies with live rates · investments and PAC tracker · Year Overview with charts.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="C16" s="9" t="inlineStr">
+    <row r="22">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>https://carloludovicocapizzoto.github.io/quadro/</t>
         </is>
@@ -1022,12 +1076,16 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="9611"/>
-  <mergeCells count="6">
+  <mergeCells count="10">
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C16:D16"/>
     <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C17:D17"/>
     <mergeCell ref="C8:D8"/>
   </mergeCells>
   <dataValidations count="1">
@@ -1036,7 +1094,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1091,12 +1149,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Budget year</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="12" t="n">
         <v>2026</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -1116,12 +1174,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Month starts on day</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1146,12 +1204,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Your currency</t>
         </is>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="13">
         <f>IFERROR(INDEX($O$4:$O$29,MATCH('Start Here'!$C$5,$N$4:$N$29,0)),"EUR")</f>
         <v/>
       </c>
@@ -1177,12 +1235,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Month to track (1-12)</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="12" t="n">
         <v>1</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -1241,17 +1299,17 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Share of income</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Starting balance</t>
         </is>
@@ -1273,18 +1331,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>0.55</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="17">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>55-20-15-10 is the split I recommend, not a must: set the percentages that fit your life.</t>
+        </is>
+      </c>
+      <c r="K11" s="18">
         <f>B11</f>
         <v/>
       </c>
@@ -1305,18 +1368,23 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="17">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>You can also rename the buckets. Only rule: the shares add up to 100%.</t>
+        </is>
+      </c>
+      <c r="K12" s="18">
         <f>B12</f>
         <v/>
       </c>
@@ -1337,18 +1405,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="17">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Tip: give each bucket its own pocket or account at your bank (see Start Here).</t>
+        </is>
+      </c>
+      <c r="K13" s="18">
         <f>B13</f>
         <v/>
       </c>
@@ -1369,18 +1442,18 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="17">
+      <c r="K14" s="18">
         <f>B14</f>
         <v/>
       </c>
@@ -1401,16 +1474,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="19">
         <f>SUM(C11:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="20">
         <f>IF(ROUND(C15,4)=1,"✓ Adds up to 100%","⚠ Must add up to 100%")</f>
         <v/>
       </c>
@@ -1475,17 +1548,17 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Default bucket</t>
         </is>
@@ -1502,35 +1575,35 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Salary</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n"/>
+      <c r="D19" s="15" t="n"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Income: money in · Expense: spending · Saving: money set aside (counts against its bucket, not as spending)</t>
         </is>
       </c>
-      <c r="H19" s="17">
+      <c r="H19" s="18">
         <f>IF(B19="","",COUNTIF($B$19:B19,"?*"))</f>
         <v/>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(1,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(1,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L19" s="17">
+      <c r="L19" s="18">
         <f>IF(OR(B19="",C19="Income"),"",SUMPRODUCT(($B$19:B19&lt;&gt;"")*($C$19:C19&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1546,30 +1619,30 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Extra Income</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D20" s="14" t="n"/>
-      <c r="H20" s="17">
+      <c r="D20" s="15" t="n"/>
+      <c r="H20" s="18">
         <f>IF(B20="","",COUNTIF($B$19:B20,"?*"))</f>
         <v/>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(2,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(2,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L20" s="17">
+      <c r="L20" s="18">
         <f>IF(OR(B20="",C20="Income"),"",SUMPRODUCT(($B$19:B20&lt;&gt;"")*($C$19:C20&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1585,34 +1658,34 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Fixed Costs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="18">
         <f>IF(B21="","",COUNTIF($B$19:B21,"?*"))</f>
         <v/>
       </c>
-      <c r="I21" s="17">
+      <c r="I21" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(3,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J21" s="17">
+      <c r="J21" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(3,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L21" s="17">
+      <c r="L21" s="18">
         <f>IF(OR(B21="",C21="Income"),"",SUMPRODUCT(($B$19:B21&lt;&gt;"")*($C$19:C21&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1628,34 +1701,34 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Groceries</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H22" s="17">
+      <c r="H22" s="18">
         <f>IF(B22="","",COUNTIF($B$19:B22,"?*"))</f>
         <v/>
       </c>
-      <c r="I22" s="17">
+      <c r="I22" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(4,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J22" s="17">
+      <c r="J22" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(4,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L22" s="17">
+      <c r="L22" s="18">
         <f>IF(OR(B22="",C22="Income"),"",SUMPRODUCT(($B$19:B22&lt;&gt;"")*($C$19:C22&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1671,34 +1744,34 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H23" s="17">
+      <c r="H23" s="18">
         <f>IF(B23="","",COUNTIF($B$19:B23,"?*"))</f>
         <v/>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(5,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J23" s="17">
+      <c r="J23" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(5,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L23" s="17">
+      <c r="L23" s="18">
         <f>IF(OR(B23="",C23="Income"),"",SUMPRODUCT(($B$19:B23&lt;&gt;"")*($C$19:C23&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1714,34 +1787,34 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H24" s="17">
+      <c r="H24" s="18">
         <f>IF(B24="","",COUNTIF($B$19:B24,"?*"))</f>
         <v/>
       </c>
-      <c r="I24" s="17">
+      <c r="I24" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(6,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J24" s="17">
+      <c r="J24" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(6,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L24" s="17">
+      <c r="L24" s="18">
         <f>IF(OR(B24="",C24="Income"),"",SUMPRODUCT(($B$19:B24&lt;&gt;"")*($C$19:C24&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1757,34 +1830,34 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Eating Out</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H25" s="17">
+      <c r="H25" s="18">
         <f>IF(B25="","",COUNTIF($B$19:B25,"?*"))</f>
         <v/>
       </c>
-      <c r="I25" s="17">
+      <c r="I25" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(7,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J25" s="17">
+      <c r="J25" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(7,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L25" s="17">
+      <c r="L25" s="18">
         <f>IF(OR(B25="",C25="Income"),"",SUMPRODUCT(($B$19:B25&lt;&gt;"")*($C$19:C25&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1800,34 +1873,34 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Fun &amp; Shopping</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H26" s="17">
+      <c r="H26" s="18">
         <f>IF(B26="","",COUNTIF($B$19:B26,"?*"))</f>
         <v/>
       </c>
-      <c r="I26" s="17">
+      <c r="I26" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(8,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J26" s="17">
+      <c r="J26" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(8,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L26" s="17">
+      <c r="L26" s="18">
         <f>IF(OR(B26="",C26="Income"),"",SUMPRODUCT(($B$19:B26&lt;&gt;"")*($C$19:C26&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1843,34 +1916,34 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Gifts</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H27" s="17">
+      <c r="H27" s="18">
         <f>IF(B27="","",COUNTIF($B$19:B27,"?*"))</f>
         <v/>
       </c>
-      <c r="I27" s="17">
+      <c r="I27" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(9,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J27" s="17">
+      <c r="J27" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(9,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L27" s="17">
+      <c r="L27" s="18">
         <f>IF(OR(B27="",C27="Income"),"",SUMPRODUCT(($B$19:B27&lt;&gt;"")*($C$19:C27&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1886,34 +1959,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H28" s="17">
+      <c r="H28" s="18">
         <f>IF(B28="","",COUNTIF($B$19:B28,"?*"))</f>
         <v/>
       </c>
-      <c r="I28" s="17">
+      <c r="I28" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(10,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J28" s="17">
+      <c r="J28" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(10,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L28" s="17">
+      <c r="L28" s="18">
         <f>IF(OR(B28="",C28="Income"),"",SUMPRODUCT(($B$19:B28&lt;&gt;"")*($C$19:C28&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1929,34 +2002,34 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Saving</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="H29" s="17">
+      <c r="H29" s="18">
         <f>IF(B29="","",COUNTIF($B$19:B29,"?*"))</f>
         <v/>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(11,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J29" s="17">
+      <c r="J29" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(11,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L29" s="17">
+      <c r="L29" s="18">
         <f>IF(OR(B29="",C29="Income"),"",SUMPRODUCT(($B$19:B29&lt;&gt;"")*($C$19:C29&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1972,202 +2045,202 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Saving</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="H30" s="17">
+      <c r="H30" s="18">
         <f>IF(B30="","",COUNTIF($B$19:B30,"?*"))</f>
         <v/>
       </c>
-      <c r="I30" s="17">
+      <c r="I30" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(12,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J30" s="17">
+      <c r="J30" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(12,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L30" s="17">
+      <c r="L30" s="18">
         <f>IF(OR(B30="",C30="Income"),"",SUMPRODUCT(($B$19:B30&lt;&gt;"")*($C$19:C30&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="H31" s="17">
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="H31" s="18">
         <f>IF(B31="","",COUNTIF($B$19:B31,"?*"))</f>
         <v/>
       </c>
-      <c r="I31" s="17">
+      <c r="I31" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(13,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J31" s="17">
+      <c r="J31" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(13,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L31" s="17">
+      <c r="L31" s="18">
         <f>IF(OR(B31="",C31="Income"),"",SUMPRODUCT(($B$19:B31&lt;&gt;"")*($C$19:C31&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="H32" s="17">
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="H32" s="18">
         <f>IF(B32="","",COUNTIF($B$19:B32,"?*"))</f>
         <v/>
       </c>
-      <c r="I32" s="17">
+      <c r="I32" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(14,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J32" s="17">
+      <c r="J32" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(14,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L32" s="17">
+      <c r="L32" s="18">
         <f>IF(OR(B32="",C32="Income"),"",SUMPRODUCT(($B$19:B32&lt;&gt;"")*($C$19:C32&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="H33" s="17">
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="H33" s="18">
         <f>IF(B33="","",COUNTIF($B$19:B33,"?*"))</f>
         <v/>
       </c>
-      <c r="I33" s="17">
+      <c r="I33" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(15,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J33" s="17">
+      <c r="J33" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(15,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L33" s="17">
+      <c r="L33" s="18">
         <f>IF(OR(B33="",C33="Income"),"",SUMPRODUCT(($B$19:B33&lt;&gt;"")*($C$19:C33&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="H34" s="17">
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="H34" s="18">
         <f>IF(B34="","",COUNTIF($B$19:B34,"?*"))</f>
         <v/>
       </c>
-      <c r="I34" s="17">
+      <c r="I34" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(16,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J34" s="17">
+      <c r="J34" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(16,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L34" s="17">
+      <c r="L34" s="18">
         <f>IF(OR(B34="",C34="Income"),"",SUMPRODUCT(($B$19:B34&lt;&gt;"")*($C$19:C34&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="H35" s="17">
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="H35" s="18">
         <f>IF(B35="","",COUNTIF($B$19:B35,"?*"))</f>
         <v/>
       </c>
-      <c r="I35" s="17">
+      <c r="I35" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(17,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J35" s="17">
+      <c r="J35" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(17,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L35" s="17">
+      <c r="L35" s="18">
         <f>IF(OR(B35="",C35="Income"),"",SUMPRODUCT(($B$19:B35&lt;&gt;"")*($C$19:C35&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="H36" s="17">
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="H36" s="18">
         <f>IF(B36="","",COUNTIF($B$19:B36,"?*"))</f>
         <v/>
       </c>
-      <c r="I36" s="17">
+      <c r="I36" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(18,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J36" s="17">
+      <c r="J36" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(18,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L36" s="17">
+      <c r="L36" s="18">
         <f>IF(OR(B36="",C36="Income"),"",SUMPRODUCT(($B$19:B36&lt;&gt;"")*($C$19:C36&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="14" t="n"/>
-      <c r="H37" s="17">
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="H37" s="18">
         <f>IF(B37="","",COUNTIF($B$19:B37,"?*"))</f>
         <v/>
       </c>
-      <c r="I37" s="17">
+      <c r="I37" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(19,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J37" s="17">
+      <c r="J37" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(19,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L37" s="17">
+      <c r="L37" s="18">
         <f>IF(OR(B37="",C37="Income"),"",SUMPRODUCT(($B$19:B37&lt;&gt;"")*($C$19:C37&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="H38" s="17">
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="H38" s="18">
         <f>IF(B38="","",COUNTIF($B$19:B38,"?*"))</f>
         <v/>
       </c>
-      <c r="I38" s="17">
+      <c r="I38" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(20,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J38" s="17">
+      <c r="J38" s="18">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(20,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L38" s="17">
+      <c r="L38" s="18">
         <f>IF(OR(B38="",C38="Income"),"",SUMPRODUCT(($B$19:B38&lt;&gt;"")*($C$19:C38&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -2281,11 +2354,11 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20">
+      <c r="A1" s="21">
         <f>INDEX({"January","February","March","April","May","June","July","August","September","October","November","December"},Settings!$C$7)</f>
         <v/>
       </c>
-      <c r="C1" s="21">
+      <c r="C1" s="22">
         <f>Settings!$C$4</f>
         <v/>
       </c>
@@ -2299,7 +2372,7 @@
           <t>Checks</t>
         </is>
       </c>
-      <c r="ZZ1" s="17">
+      <c r="ZZ1" s="18">
         <f>Settings!$C$6</f>
         <v/>
       </c>
@@ -2310,20 +2383,20 @@
           <t>Period</t>
         </is>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="23">
         <f>DATE(Settings!$C$4,Settings!$C$7-IF(Settings!$C$5=1,0,1),Settings!$C$5)</f>
         <v/>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="23">
         <f>DATE(Settings!$C$4,Settings!$C$7+1-IF(Settings!$C$5=1,0,1),Settings!$C$5)-1</f>
         <v/>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="L2" s="23">
+      <c r="L2" s="24">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income")</f>
         <v/>
       </c>
@@ -2332,18 +2405,18 @@
           <t>Missing category</t>
         </is>
       </c>
-      <c r="P2" s="24">
+      <c r="P2" s="25">
         <f>SUMPRODUCT(($D$10:$D$49&lt;&gt;"")*($C$10:$C$49=""))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="K3" s="10" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="L3" s="23">
+      <c r="L3" s="24">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Expense")</f>
         <v/>
       </c>
@@ -2352,7 +2425,7 @@
           <t>Unknown category</t>
         </is>
       </c>
-      <c r="P3" s="24">
+      <c r="P3" s="25">
         <f>COUNTIF($H$10:$H$49,"Unknown")</f>
         <v/>
       </c>
@@ -2363,12 +2436,12 @@
           <t>How to use</t>
         </is>
       </c>
-      <c r="K4" s="10" t="inlineStr">
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>Saved &amp; invested</t>
         </is>
       </c>
-      <c r="L4" s="23">
+      <c r="L4" s="24">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Saving")</f>
         <v/>
       </c>
@@ -2377,7 +2450,7 @@
           <t>Dates typed as text</t>
         </is>
       </c>
-      <c r="P4" s="24">
+      <c r="P4" s="25">
         <f>SUMPRODUCT(($A$10:$A$49&lt;&gt;"")*NOT(ISNUMBER($A$10:$A$49)))</f>
         <v/>
       </c>
@@ -2388,12 +2461,12 @@
           <t>Add one row per transaction in the yellow cells. Pick a category: bucket and type fill in by themselves.</t>
         </is>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>Left over</t>
         </is>
       </c>
-      <c r="L5" s="23">
+      <c r="L5" s="24">
         <f>L2-L3-L4</f>
         <v/>
       </c>
@@ -2402,7 +2475,7 @@
           <t>Dates outside this period</t>
         </is>
       </c>
-      <c r="P5" s="24">
+      <c r="P5" s="25">
         <f>SUMPRODUCT(ISNUMBER($A$10:$A$49)*((($A$10:$A$49&lt;$B$2)+($A$10:$A$49&gt;$C$2))&gt;0))</f>
         <v/>
       </c>
@@ -2413,7 +2486,7 @@
           <t>Paid with money from another bucket? Choose it in “Paid from / Allocate to”. For income, pick a bucket to put it all there, or leave blank to split it by your rule.</t>
         </is>
       </c>
-      <c r="N6" s="19">
+      <c r="N6" s="20">
         <f>IF(SUM(P2:P5)=0,"✓ All good","⚠ Fix the rows highlighted in red")</f>
         <v/>
       </c>
@@ -2427,358 +2500,358 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="26">
         <f>"Amount"</f>
         <v/>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Paid from / Allocate to</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="26">
         <f>"In your currency "&amp;"("&amp;Settings!$C$6&amp;")"</f>
         <v/>
       </c>
-      <c r="K9" s="13" t="inlineStr">
+      <c r="K9" s="14" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="L9" s="13" t="inlineStr">
+      <c r="L9" s="14" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="M9" s="13" t="inlineStr">
+      <c r="M9" s="14" t="inlineStr">
         <is>
           <t>Carried over</t>
         </is>
       </c>
-      <c r="N9" s="13" t="inlineStr">
+      <c r="N9" s="14" t="inlineStr">
         <is>
           <t>From income</t>
         </is>
       </c>
-      <c r="O9" s="13" t="inlineStr">
+      <c r="O9" s="14" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="P9" s="13" t="inlineStr">
+      <c r="P9" s="14" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="14" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="28">
+      <c r="A10" s="27" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="28" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="29">
         <f>IF(C10="","",IF(H10="Income",IF(F10="","Split by rule",F10),IF(OR(F10="",F10="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C10,Settings!$B$19:$B$38,0)),""),F10)))</f>
         <v/>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="29">
         <f>IF(C10="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C10,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I10" s="29">
+      <c r="I10" s="30">
         <f>IF(D10="","",D10)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>Settings!$B$11</f>
         <v/>
       </c>
-      <c r="L10" s="31">
+      <c r="L10" s="32">
         <f>Settings!$C$11</f>
         <v/>
       </c>
-      <c r="M10" s="32">
+      <c r="M10" s="33">
         <f>Settings!$D$11</f>
         <v/>
       </c>
-      <c r="N10" s="32">
+      <c r="N10" s="33">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L10+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K10)</f>
         <v/>
       </c>
-      <c r="O10" s="32">
+      <c r="O10" s="33">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K10,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P10" s="33">
+      <c r="P10" s="34">
         <f>M10+N10-O10</f>
         <v/>
       </c>
-      <c r="Q10" s="32">
+      <c r="Q10" s="33">
         <f>M10+N10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="28">
+      <c r="A11" s="27" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="28" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="29">
         <f>IF(C11="","",IF(H11="Income",IF(F11="","Split by rule",F11),IF(OR(F11="",F11="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C11,Settings!$B$19:$B$38,0)),""),F11)))</f>
         <v/>
       </c>
-      <c r="H11" s="28">
+      <c r="H11" s="29">
         <f>IF(C11="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C11,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I11" s="29">
+      <c r="I11" s="30">
         <f>IF(D11="","",D11)</f>
         <v/>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="31">
         <f>Settings!$B$12</f>
         <v/>
       </c>
-      <c r="L11" s="31">
+      <c r="L11" s="32">
         <f>Settings!$C$12</f>
         <v/>
       </c>
-      <c r="M11" s="32">
+      <c r="M11" s="33">
         <f>Settings!$D$12</f>
         <v/>
       </c>
-      <c r="N11" s="32">
+      <c r="N11" s="33">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L11+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K11)</f>
         <v/>
       </c>
-      <c r="O11" s="32">
+      <c r="O11" s="33">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K11,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P11" s="33">
+      <c r="P11" s="34">
         <f>M11+N11-O11</f>
         <v/>
       </c>
-      <c r="Q11" s="32">
+      <c r="Q11" s="33">
         <f>M11+N11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="28">
+      <c r="A12" s="27" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="28" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="29">
         <f>IF(C12="","",IF(H12="Income",IF(F12="","Split by rule",F12),IF(OR(F12="",F12="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C12,Settings!$B$19:$B$38,0)),""),F12)))</f>
         <v/>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="29">
         <f>IF(C12="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C12,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I12" s="29">
+      <c r="I12" s="30">
         <f>IF(D12="","",D12)</f>
         <v/>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="31">
         <f>Settings!$B$13</f>
         <v/>
       </c>
-      <c r="L12" s="31">
+      <c r="L12" s="32">
         <f>Settings!$C$13</f>
         <v/>
       </c>
-      <c r="M12" s="32">
+      <c r="M12" s="33">
         <f>Settings!$D$13</f>
         <v/>
       </c>
-      <c r="N12" s="32">
+      <c r="N12" s="33">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L12+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K12)</f>
         <v/>
       </c>
-      <c r="O12" s="32">
+      <c r="O12" s="33">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K12,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P12" s="33">
+      <c r="P12" s="34">
         <f>M12+N12-O12</f>
         <v/>
       </c>
-      <c r="Q12" s="32">
+      <c r="Q12" s="33">
         <f>M12+N12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="n"/>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="28">
+      <c r="A13" s="27" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="29">
         <f>IF(C13="","",IF(H13="Income",IF(F13="","Split by rule",F13),IF(OR(F13="",F13="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C13,Settings!$B$19:$B$38,0)),""),F13)))</f>
         <v/>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="29">
         <f>IF(C13="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C13,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I13" s="29">
+      <c r="I13" s="30">
         <f>IF(D13="","",D13)</f>
         <v/>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="31">
         <f>Settings!$B$14</f>
         <v/>
       </c>
-      <c r="L13" s="31">
+      <c r="L13" s="32">
         <f>Settings!$C$14</f>
         <v/>
       </c>
-      <c r="M13" s="32">
+      <c r="M13" s="33">
         <f>Settings!$D$14</f>
         <v/>
       </c>
-      <c r="N13" s="32">
+      <c r="N13" s="33">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L13+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K13)</f>
         <v/>
       </c>
-      <c r="O13" s="32">
+      <c r="O13" s="33">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K13,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P13" s="33">
+      <c r="P13" s="34">
         <f>M13+N13-O13</f>
         <v/>
       </c>
-      <c r="Q13" s="32">
+      <c r="Q13" s="33">
         <f>M13+N13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="n"/>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="28">
+      <c r="A14" s="27" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="28" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="29">
         <f>IF(C14="","",IF(H14="Income",IF(F14="","Split by rule",F14),IF(OR(F14="",F14="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C14,Settings!$B$19:$B$38,0)),""),F14)))</f>
         <v/>
       </c>
-      <c r="H14" s="28">
+      <c r="H14" s="29">
         <f>IF(C14="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C14,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I14" s="29">
+      <c r="I14" s="30">
         <f>IF(D14="","",D14)</f>
         <v/>
       </c>
-      <c r="K14" s="10" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M14" s="23">
+      <c r="M14" s="24">
         <f>SUM(M10:M13)</f>
         <v/>
       </c>
-      <c r="N14" s="23">
+      <c r="N14" s="24">
         <f>SUM(N10:N13)</f>
         <v/>
       </c>
-      <c r="O14" s="23">
+      <c r="O14" s="24">
         <f>SUM(O10:O13)</f>
         <v/>
       </c>
-      <c r="P14" s="23">
+      <c r="P14" s="24">
         <f>SUM(P10:P13)</f>
         <v/>
       </c>
-      <c r="Q14" s="23">
+      <c r="Q14" s="24">
         <f>SUM(Q10:Q13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="28">
+      <c r="A15" s="27" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="28" t="n"/>
+      <c r="E15" s="15" t="n"/>
+      <c r="F15" s="15" t="n"/>
+      <c r="G15" s="29">
         <f>IF(C15="","",IF(H15="Income",IF(F15="","Split by rule",F15),IF(OR(F15="",F15="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C15,Settings!$B$19:$B$38,0)),""),F15)))</f>
         <v/>
       </c>
-      <c r="H15" s="28">
+      <c r="H15" s="29">
         <f>IF(C15="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C15,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I15" s="29">
+      <c r="I15" s="30">
         <f>IF(D15="","",D15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="26" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="28">
+      <c r="A16" s="27" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="28" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="29">
         <f>IF(C16="","",IF(H16="Income",IF(F16="","Split by rule",F16),IF(OR(F16="",F16="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C16,Settings!$B$19:$B$38,0)),""),F16)))</f>
         <v/>
       </c>
-      <c r="H16" s="28">
+      <c r="H16" s="29">
         <f>IF(C16="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C16,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I16" s="29">
+      <c r="I16" s="30">
         <f>IF(D16="","",D16)</f>
         <v/>
       </c>
@@ -2789,925 +2862,925 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="26" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="27" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="28">
+      <c r="A17" s="27" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="28" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="29">
         <f>IF(C17="","",IF(H17="Income",IF(F17="","Split by rule",F17),IF(OR(F17="",F17="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C17,Settings!$B$19:$B$38,0)),""),F17)))</f>
         <v/>
       </c>
-      <c r="H17" s="28">
+      <c r="H17" s="29">
         <f>IF(C17="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C17,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I17" s="29">
+      <c r="I17" s="30">
         <f>IF(D17="","",D17)</f>
         <v/>
       </c>
-      <c r="K17" s="13" t="inlineStr">
+      <c r="K17" s="14" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="L17" s="13" t="inlineStr">
+      <c r="L17" s="14" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="M17" s="13" t="inlineStr">
+      <c r="M17" s="14" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="n"/>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="28">
+      <c r="A18" s="27" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="28" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="29">
         <f>IF(C18="","",IF(H18="Income",IF(F18="","Split by rule",F18),IF(OR(F18="",F18="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C18,Settings!$B$19:$B$38,0)),""),F18)))</f>
         <v/>
       </c>
-      <c r="H18" s="28">
+      <c r="H18" s="29">
         <f>IF(C18="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C18,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I18" s="29">
+      <c r="I18" s="30">
         <f>IF(D18="","",D18)</f>
         <v/>
       </c>
-      <c r="K18" s="34">
+      <c r="K18" s="35">
         <f>Settings!$J$19</f>
         <v/>
       </c>
-      <c r="L18" s="32">
+      <c r="L18" s="33">
         <f>IF(K18="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K18))</f>
         <v/>
       </c>
-      <c r="M18" s="35">
+      <c r="M18" s="36">
         <f>IF(OR(K18="",L38=0),"",L18/L38)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="26" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="27" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="28">
+      <c r="A19" s="27" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="29">
         <f>IF(C19="","",IF(H19="Income",IF(F19="","Split by rule",F19),IF(OR(F19="",F19="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C19,Settings!$B$19:$B$38,0)),""),F19)))</f>
         <v/>
       </c>
-      <c r="H19" s="28">
+      <c r="H19" s="29">
         <f>IF(C19="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C19,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I19" s="29">
+      <c r="I19" s="30">
         <f>IF(D19="","",D19)</f>
         <v/>
       </c>
-      <c r="K19" s="34">
+      <c r="K19" s="35">
         <f>Settings!$J$20</f>
         <v/>
       </c>
-      <c r="L19" s="32">
+      <c r="L19" s="33">
         <f>IF(K19="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K19))</f>
         <v/>
       </c>
-      <c r="M19" s="35">
+      <c r="M19" s="36">
         <f>IF(OR(K19="",L38=0),"",L19/L38)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="26" t="n"/>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="27" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="28">
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="28" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="29">
         <f>IF(C20="","",IF(H20="Income",IF(F20="","Split by rule",F20),IF(OR(F20="",F20="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C20,Settings!$B$19:$B$38,0)),""),F20)))</f>
         <v/>
       </c>
-      <c r="H20" s="28">
+      <c r="H20" s="29">
         <f>IF(C20="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C20,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I20" s="29">
+      <c r="I20" s="30">
         <f>IF(D20="","",D20)</f>
         <v/>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="35">
         <f>Settings!$J$21</f>
         <v/>
       </c>
-      <c r="L20" s="32">
+      <c r="L20" s="33">
         <f>IF(K20="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K20))</f>
         <v/>
       </c>
-      <c r="M20" s="35">
+      <c r="M20" s="36">
         <f>IF(OR(K20="",L38=0),"",L20/L38)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="26" t="n"/>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="27" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="28">
+      <c r="A21" s="27" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="28" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="29">
         <f>IF(C21="","",IF(H21="Income",IF(F21="","Split by rule",F21),IF(OR(F21="",F21="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C21,Settings!$B$19:$B$38,0)),""),F21)))</f>
         <v/>
       </c>
-      <c r="H21" s="28">
+      <c r="H21" s="29">
         <f>IF(C21="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C21,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I21" s="29">
+      <c r="I21" s="30">
         <f>IF(D21="","",D21)</f>
         <v/>
       </c>
-      <c r="K21" s="34">
+      <c r="K21" s="35">
         <f>Settings!$J$22</f>
         <v/>
       </c>
-      <c r="L21" s="32">
+      <c r="L21" s="33">
         <f>IF(K21="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K21))</f>
         <v/>
       </c>
-      <c r="M21" s="35">
+      <c r="M21" s="36">
         <f>IF(OR(K21="",L38=0),"",L21/L38)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="26" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="27" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="28">
+      <c r="A22" s="27" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="28" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="29">
         <f>IF(C22="","",IF(H22="Income",IF(F22="","Split by rule",F22),IF(OR(F22="",F22="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C22,Settings!$B$19:$B$38,0)),""),F22)))</f>
         <v/>
       </c>
-      <c r="H22" s="28">
+      <c r="H22" s="29">
         <f>IF(C22="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C22,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I22" s="29">
+      <c r="I22" s="30">
         <f>IF(D22="","",D22)</f>
         <v/>
       </c>
-      <c r="K22" s="34">
+      <c r="K22" s="35">
         <f>Settings!$J$23</f>
         <v/>
       </c>
-      <c r="L22" s="32">
+      <c r="L22" s="33">
         <f>IF(K22="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K22))</f>
         <v/>
       </c>
-      <c r="M22" s="35">
+      <c r="M22" s="36">
         <f>IF(OR(K22="",L38=0),"",L22/L38)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="26" t="n"/>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="27" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="28">
+      <c r="A23" s="27" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="28" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="29">
         <f>IF(C23="","",IF(H23="Income",IF(F23="","Split by rule",F23),IF(OR(F23="",F23="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C23,Settings!$B$19:$B$38,0)),""),F23)))</f>
         <v/>
       </c>
-      <c r="H23" s="28">
+      <c r="H23" s="29">
         <f>IF(C23="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C23,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I23" s="29">
+      <c r="I23" s="30">
         <f>IF(D23="","",D23)</f>
         <v/>
       </c>
-      <c r="K23" s="34">
+      <c r="K23" s="35">
         <f>Settings!$J$24</f>
         <v/>
       </c>
-      <c r="L23" s="32">
+      <c r="L23" s="33">
         <f>IF(K23="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K23))</f>
         <v/>
       </c>
-      <c r="M23" s="35">
+      <c r="M23" s="36">
         <f>IF(OR(K23="",L38=0),"",L23/L38)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="n"/>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="27" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="28">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="28" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="29">
         <f>IF(C24="","",IF(H24="Income",IF(F24="","Split by rule",F24),IF(OR(F24="",F24="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C24,Settings!$B$19:$B$38,0)),""),F24)))</f>
         <v/>
       </c>
-      <c r="H24" s="28">
+      <c r="H24" s="29">
         <f>IF(C24="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C24,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I24" s="29">
+      <c r="I24" s="30">
         <f>IF(D24="","",D24)</f>
         <v/>
       </c>
-      <c r="K24" s="34">
+      <c r="K24" s="35">
         <f>Settings!$J$25</f>
         <v/>
       </c>
-      <c r="L24" s="32">
+      <c r="L24" s="33">
         <f>IF(K24="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K24))</f>
         <v/>
       </c>
-      <c r="M24" s="35">
+      <c r="M24" s="36">
         <f>IF(OR(K24="",L38=0),"",L24/L38)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="n"/>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="27" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="28">
+      <c r="A25" s="27" t="n"/>
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="28" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="29">
         <f>IF(C25="","",IF(H25="Income",IF(F25="","Split by rule",F25),IF(OR(F25="",F25="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C25,Settings!$B$19:$B$38,0)),""),F25)))</f>
         <v/>
       </c>
-      <c r="H25" s="28">
+      <c r="H25" s="29">
         <f>IF(C25="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C25,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I25" s="29">
+      <c r="I25" s="30">
         <f>IF(D25="","",D25)</f>
         <v/>
       </c>
-      <c r="K25" s="34">
+      <c r="K25" s="35">
         <f>Settings!$J$26</f>
         <v/>
       </c>
-      <c r="L25" s="32">
+      <c r="L25" s="33">
         <f>IF(K25="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K25))</f>
         <v/>
       </c>
-      <c r="M25" s="35">
+      <c r="M25" s="36">
         <f>IF(OR(K25="",L38=0),"",L25/L38)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="n"/>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="28">
+      <c r="A26" s="27" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="28" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="29">
         <f>IF(C26="","",IF(H26="Income",IF(F26="","Split by rule",F26),IF(OR(F26="",F26="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C26,Settings!$B$19:$B$38,0)),""),F26)))</f>
         <v/>
       </c>
-      <c r="H26" s="28">
+      <c r="H26" s="29">
         <f>IF(C26="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C26,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I26" s="29">
+      <c r="I26" s="30">
         <f>IF(D26="","",D26)</f>
         <v/>
       </c>
-      <c r="K26" s="34">
+      <c r="K26" s="35">
         <f>Settings!$J$27</f>
         <v/>
       </c>
-      <c r="L26" s="32">
+      <c r="L26" s="33">
         <f>IF(K26="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K26))</f>
         <v/>
       </c>
-      <c r="M26" s="35">
+      <c r="M26" s="36">
         <f>IF(OR(K26="",L38=0),"",L26/L38)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="26" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="27" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="28">
+      <c r="A27" s="27" t="n"/>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="28" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="29">
         <f>IF(C27="","",IF(H27="Income",IF(F27="","Split by rule",F27),IF(OR(F27="",F27="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C27,Settings!$B$19:$B$38,0)),""),F27)))</f>
         <v/>
       </c>
-      <c r="H27" s="28">
+      <c r="H27" s="29">
         <f>IF(C27="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C27,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I27" s="29">
+      <c r="I27" s="30">
         <f>IF(D27="","",D27)</f>
         <v/>
       </c>
-      <c r="K27" s="34">
+      <c r="K27" s="35">
         <f>Settings!$J$28</f>
         <v/>
       </c>
-      <c r="L27" s="32">
+      <c r="L27" s="33">
         <f>IF(K27="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K27))</f>
         <v/>
       </c>
-      <c r="M27" s="35">
+      <c r="M27" s="36">
         <f>IF(OR(K27="",L38=0),"",L27/L38)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="26" t="n"/>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="28">
+      <c r="A28" s="27" t="n"/>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="28" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="29">
         <f>IF(C28="","",IF(H28="Income",IF(F28="","Split by rule",F28),IF(OR(F28="",F28="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C28,Settings!$B$19:$B$38,0)),""),F28)))</f>
         <v/>
       </c>
-      <c r="H28" s="28">
+      <c r="H28" s="29">
         <f>IF(C28="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C28,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I28" s="29">
+      <c r="I28" s="30">
         <f>IF(D28="","",D28)</f>
         <v/>
       </c>
-      <c r="K28" s="34">
+      <c r="K28" s="35">
         <f>Settings!$J$29</f>
         <v/>
       </c>
-      <c r="L28" s="32">
+      <c r="L28" s="33">
         <f>IF(K28="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K28))</f>
         <v/>
       </c>
-      <c r="M28" s="35">
+      <c r="M28" s="36">
         <f>IF(OR(K28="",L38=0),"",L28/L38)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="26" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="27" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="28">
+      <c r="A29" s="27" t="n"/>
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="28" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="29">
         <f>IF(C29="","",IF(H29="Income",IF(F29="","Split by rule",F29),IF(OR(F29="",F29="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C29,Settings!$B$19:$B$38,0)),""),F29)))</f>
         <v/>
       </c>
-      <c r="H29" s="28">
+      <c r="H29" s="29">
         <f>IF(C29="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C29,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I29" s="29">
+      <c r="I29" s="30">
         <f>IF(D29="","",D29)</f>
         <v/>
       </c>
-      <c r="K29" s="34">
+      <c r="K29" s="35">
         <f>Settings!$J$30</f>
         <v/>
       </c>
-      <c r="L29" s="32">
+      <c r="L29" s="33">
         <f>IF(K29="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K29))</f>
         <v/>
       </c>
-      <c r="M29" s="35">
+      <c r="M29" s="36">
         <f>IF(OR(K29="",L38=0),"",L29/L38)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="26" t="n"/>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="28">
+      <c r="A30" s="27" t="n"/>
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="28" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="n"/>
+      <c r="G30" s="29">
         <f>IF(C30="","",IF(H30="Income",IF(F30="","Split by rule",F30),IF(OR(F30="",F30="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C30,Settings!$B$19:$B$38,0)),""),F30)))</f>
         <v/>
       </c>
-      <c r="H30" s="28">
+      <c r="H30" s="29">
         <f>IF(C30="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C30,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I30" s="29">
+      <c r="I30" s="30">
         <f>IF(D30="","",D30)</f>
         <v/>
       </c>
-      <c r="K30" s="34">
+      <c r="K30" s="35">
         <f>Settings!$J$31</f>
         <v/>
       </c>
-      <c r="L30" s="32">
+      <c r="L30" s="33">
         <f>IF(K30="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K30))</f>
         <v/>
       </c>
-      <c r="M30" s="35">
+      <c r="M30" s="36">
         <f>IF(OR(K30="",L38=0),"",L30/L38)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="26" t="n"/>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="27" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="28">
+      <c r="A31" s="27" t="n"/>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="28" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
+      <c r="G31" s="29">
         <f>IF(C31="","",IF(H31="Income",IF(F31="","Split by rule",F31),IF(OR(F31="",F31="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C31,Settings!$B$19:$B$38,0)),""),F31)))</f>
         <v/>
       </c>
-      <c r="H31" s="28">
+      <c r="H31" s="29">
         <f>IF(C31="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C31,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I31" s="29">
+      <c r="I31" s="30">
         <f>IF(D31="","",D31)</f>
         <v/>
       </c>
-      <c r="K31" s="34">
+      <c r="K31" s="35">
         <f>Settings!$J$32</f>
         <v/>
       </c>
-      <c r="L31" s="32">
+      <c r="L31" s="33">
         <f>IF(K31="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K31))</f>
         <v/>
       </c>
-      <c r="M31" s="35">
+      <c r="M31" s="36">
         <f>IF(OR(K31="",L38=0),"",L31/L38)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="n"/>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="27" t="n"/>
-      <c r="E32" s="14" t="n"/>
-      <c r="F32" s="14" t="n"/>
-      <c r="G32" s="28">
+      <c r="A32" s="27" t="n"/>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="28" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="29">
         <f>IF(C32="","",IF(H32="Income",IF(F32="","Split by rule",F32),IF(OR(F32="",F32="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C32,Settings!$B$19:$B$38,0)),""),F32)))</f>
         <v/>
       </c>
-      <c r="H32" s="28">
+      <c r="H32" s="29">
         <f>IF(C32="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C32,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I32" s="29">
+      <c r="I32" s="30">
         <f>IF(D32="","",D32)</f>
         <v/>
       </c>
-      <c r="K32" s="34">
+      <c r="K32" s="35">
         <f>Settings!$J$33</f>
         <v/>
       </c>
-      <c r="L32" s="32">
+      <c r="L32" s="33">
         <f>IF(K32="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K32))</f>
         <v/>
       </c>
-      <c r="M32" s="35">
+      <c r="M32" s="36">
         <f>IF(OR(K32="",L38=0),"",L32/L38)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="26" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="27" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="28">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="28" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="29">
         <f>IF(C33="","",IF(H33="Income",IF(F33="","Split by rule",F33),IF(OR(F33="",F33="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C33,Settings!$B$19:$B$38,0)),""),F33)))</f>
         <v/>
       </c>
-      <c r="H33" s="28">
+      <c r="H33" s="29">
         <f>IF(C33="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C33,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I33" s="29">
+      <c r="I33" s="30">
         <f>IF(D33="","",D33)</f>
         <v/>
       </c>
-      <c r="K33" s="34">
+      <c r="K33" s="35">
         <f>Settings!$J$34</f>
         <v/>
       </c>
-      <c r="L33" s="32">
+      <c r="L33" s="33">
         <f>IF(K33="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K33))</f>
         <v/>
       </c>
-      <c r="M33" s="35">
+      <c r="M33" s="36">
         <f>IF(OR(K33="",L38=0),"",L33/L38)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="26" t="n"/>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="27" t="n"/>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="28">
+      <c r="A34" s="27" t="n"/>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="28" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="29">
         <f>IF(C34="","",IF(H34="Income",IF(F34="","Split by rule",F34),IF(OR(F34="",F34="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C34,Settings!$B$19:$B$38,0)),""),F34)))</f>
         <v/>
       </c>
-      <c r="H34" s="28">
+      <c r="H34" s="29">
         <f>IF(C34="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C34,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I34" s="29">
+      <c r="I34" s="30">
         <f>IF(D34="","",D34)</f>
         <v/>
       </c>
-      <c r="K34" s="34">
+      <c r="K34" s="35">
         <f>Settings!$J$35</f>
         <v/>
       </c>
-      <c r="L34" s="32">
+      <c r="L34" s="33">
         <f>IF(K34="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K34))</f>
         <v/>
       </c>
-      <c r="M34" s="35">
+      <c r="M34" s="36">
         <f>IF(OR(K34="",L38=0),"",L34/L38)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="26" t="n"/>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="27" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="14" t="n"/>
-      <c r="G35" s="28">
+      <c r="A35" s="27" t="n"/>
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="28" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="29">
         <f>IF(C35="","",IF(H35="Income",IF(F35="","Split by rule",F35),IF(OR(F35="",F35="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C35,Settings!$B$19:$B$38,0)),""),F35)))</f>
         <v/>
       </c>
-      <c r="H35" s="28">
+      <c r="H35" s="29">
         <f>IF(C35="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C35,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I35" s="29">
+      <c r="I35" s="30">
         <f>IF(D35="","",D35)</f>
         <v/>
       </c>
-      <c r="K35" s="34">
+      <c r="K35" s="35">
         <f>Settings!$J$36</f>
         <v/>
       </c>
-      <c r="L35" s="32">
+      <c r="L35" s="33">
         <f>IF(K35="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K35))</f>
         <v/>
       </c>
-      <c r="M35" s="35">
+      <c r="M35" s="36">
         <f>IF(OR(K35="",L38=0),"",L35/L38)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="26" t="n"/>
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="14" t="n"/>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="28">
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="15" t="n"/>
+      <c r="F36" s="15" t="n"/>
+      <c r="G36" s="29">
         <f>IF(C36="","",IF(H36="Income",IF(F36="","Split by rule",F36),IF(OR(F36="",F36="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C36,Settings!$B$19:$B$38,0)),""),F36)))</f>
         <v/>
       </c>
-      <c r="H36" s="28">
+      <c r="H36" s="29">
         <f>IF(C36="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C36,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I36" s="29">
+      <c r="I36" s="30">
         <f>IF(D36="","",D36)</f>
         <v/>
       </c>
-      <c r="K36" s="34">
+      <c r="K36" s="35">
         <f>Settings!$J$37</f>
         <v/>
       </c>
-      <c r="L36" s="32">
+      <c r="L36" s="33">
         <f>IF(K36="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K36))</f>
         <v/>
       </c>
-      <c r="M36" s="35">
+      <c r="M36" s="36">
         <f>IF(OR(K36="",L38=0),"",L36/L38)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="26" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="27" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
-      <c r="G37" s="28">
+      <c r="A37" s="27" t="n"/>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="28" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="29">
         <f>IF(C37="","",IF(H37="Income",IF(F37="","Split by rule",F37),IF(OR(F37="",F37="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C37,Settings!$B$19:$B$38,0)),""),F37)))</f>
         <v/>
       </c>
-      <c r="H37" s="28">
+      <c r="H37" s="29">
         <f>IF(C37="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C37,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I37" s="29">
+      <c r="I37" s="30">
         <f>IF(D37="","",D37)</f>
         <v/>
       </c>
-      <c r="K37" s="34">
+      <c r="K37" s="35">
         <f>Settings!$J$38</f>
         <v/>
       </c>
-      <c r="L37" s="32">
+      <c r="L37" s="33">
         <f>IF(K37="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K37))</f>
         <v/>
       </c>
-      <c r="M37" s="35">
+      <c r="M37" s="36">
         <f>IF(OR(K37="",L38=0),"",L37/L38)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="26" t="n"/>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="27" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
-      <c r="G38" s="28">
+      <c r="A38" s="27" t="n"/>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="29">
         <f>IF(C38="","",IF(H38="Income",IF(F38="","Split by rule",F38),IF(OR(F38="",F38="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C38,Settings!$B$19:$B$38,0)),""),F38)))</f>
         <v/>
       </c>
-      <c r="H38" s="28">
+      <c r="H38" s="29">
         <f>IF(C38="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C38,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I38" s="29">
+      <c r="I38" s="30">
         <f>IF(D38="","",D38)</f>
         <v/>
       </c>
-      <c r="K38" s="10" t="inlineStr">
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="L38" s="23">
+      <c r="L38" s="24">
         <f>SUM(L18:L37)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="26" t="n"/>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="27" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="28">
+      <c r="A39" s="27" t="n"/>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="28" t="n"/>
+      <c r="E39" s="15" t="n"/>
+      <c r="F39" s="15" t="n"/>
+      <c r="G39" s="29">
         <f>IF(C39="","",IF(H39="Income",IF(F39="","Split by rule",F39),IF(OR(F39="",F39="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C39,Settings!$B$19:$B$38,0)),""),F39)))</f>
         <v/>
       </c>
-      <c r="H39" s="28">
+      <c r="H39" s="29">
         <f>IF(C39="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C39,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I39" s="29">
+      <c r="I39" s="30">
         <f>IF(D39="","",D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="26" t="n"/>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
-      <c r="G40" s="28">
+      <c r="A40" s="27" t="n"/>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="28" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="15" t="n"/>
+      <c r="G40" s="29">
         <f>IF(C40="","",IF(H40="Income",IF(F40="","Split by rule",F40),IF(OR(F40="",F40="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C40,Settings!$B$19:$B$38,0)),""),F40)))</f>
         <v/>
       </c>
-      <c r="H40" s="28">
+      <c r="H40" s="29">
         <f>IF(C40="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C40,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I40" s="29">
+      <c r="I40" s="30">
         <f>IF(D40="","",D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="26" t="n"/>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="14" t="n"/>
-      <c r="G41" s="28">
+      <c r="A41" s="27" t="n"/>
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="28" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="29">
         <f>IF(C41="","",IF(H41="Income",IF(F41="","Split by rule",F41),IF(OR(F41="",F41="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C41,Settings!$B$19:$B$38,0)),""),F41)))</f>
         <v/>
       </c>
-      <c r="H41" s="28">
+      <c r="H41" s="29">
         <f>IF(C41="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C41,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I41" s="29">
+      <c r="I41" s="30">
         <f>IF(D41="","",D41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="26" t="n"/>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="27" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="14" t="n"/>
-      <c r="G42" s="28">
+      <c r="A42" s="27" t="n"/>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="28" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="29">
         <f>IF(C42="","",IF(H42="Income",IF(F42="","Split by rule",F42),IF(OR(F42="",F42="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C42,Settings!$B$19:$B$38,0)),""),F42)))</f>
         <v/>
       </c>
-      <c r="H42" s="28">
+      <c r="H42" s="29">
         <f>IF(C42="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C42,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I42" s="29">
+      <c r="I42" s="30">
         <f>IF(D42="","",D42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="26" t="n"/>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="14" t="n"/>
-      <c r="D43" s="27" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="14" t="n"/>
-      <c r="G43" s="28">
+      <c r="A43" s="27" t="n"/>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="28" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="29">
         <f>IF(C43="","",IF(H43="Income",IF(F43="","Split by rule",F43),IF(OR(F43="",F43="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C43,Settings!$B$19:$B$38,0)),""),F43)))</f>
         <v/>
       </c>
-      <c r="H43" s="28">
+      <c r="H43" s="29">
         <f>IF(C43="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C43,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I43" s="29">
+      <c r="I43" s="30">
         <f>IF(D43="","",D43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="26" t="n"/>
-      <c r="B44" s="14" t="n"/>
-      <c r="C44" s="14" t="n"/>
-      <c r="D44" s="27" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="14" t="n"/>
-      <c r="G44" s="28">
+      <c r="A44" s="27" t="n"/>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="28" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="29">
         <f>IF(C44="","",IF(H44="Income",IF(F44="","Split by rule",F44),IF(OR(F44="",F44="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C44,Settings!$B$19:$B$38,0)),""),F44)))</f>
         <v/>
       </c>
-      <c r="H44" s="28">
+      <c r="H44" s="29">
         <f>IF(C44="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C44,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I44" s="29">
+      <c r="I44" s="30">
         <f>IF(D44="","",D44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="26" t="n"/>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="28">
+      <c r="A45" s="27" t="n"/>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="28" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="29">
         <f>IF(C45="","",IF(H45="Income",IF(F45="","Split by rule",F45),IF(OR(F45="",F45="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C45,Settings!$B$19:$B$38,0)),""),F45)))</f>
         <v/>
       </c>
-      <c r="H45" s="28">
+      <c r="H45" s="29">
         <f>IF(C45="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C45,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I45" s="29">
+      <c r="I45" s="30">
         <f>IF(D45="","",D45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="26" t="n"/>
-      <c r="B46" s="14" t="n"/>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="27" t="n"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="14" t="n"/>
-      <c r="G46" s="28">
+      <c r="A46" s="27" t="n"/>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="28" t="n"/>
+      <c r="E46" s="15" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="29">
         <f>IF(C46="","",IF(H46="Income",IF(F46="","Split by rule",F46),IF(OR(F46="",F46="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C46,Settings!$B$19:$B$38,0)),""),F46)))</f>
         <v/>
       </c>
-      <c r="H46" s="28">
+      <c r="H46" s="29">
         <f>IF(C46="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C46,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I46" s="29">
+      <c r="I46" s="30">
         <f>IF(D46="","",D46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="26" t="n"/>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="28">
+      <c r="A47" s="27" t="n"/>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="28" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="29">
         <f>IF(C47="","",IF(H47="Income",IF(F47="","Split by rule",F47),IF(OR(F47="",F47="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C47,Settings!$B$19:$B$38,0)),""),F47)))</f>
         <v/>
       </c>
-      <c r="H47" s="28">
+      <c r="H47" s="29">
         <f>IF(C47="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C47,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I47" s="29">
+      <c r="I47" s="30">
         <f>IF(D47="","",D47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="26" t="n"/>
-      <c r="B48" s="14" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="27" t="n"/>
-      <c r="E48" s="14" t="n"/>
-      <c r="F48" s="14" t="n"/>
-      <c r="G48" s="28">
+      <c r="A48" s="27" t="n"/>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="28" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="29">
         <f>IF(C48="","",IF(H48="Income",IF(F48="","Split by rule",F48),IF(OR(F48="",F48="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C48,Settings!$B$19:$B$38,0)),""),F48)))</f>
         <v/>
       </c>
-      <c r="H48" s="28">
+      <c r="H48" s="29">
         <f>IF(C48="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C48,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I48" s="29">
+      <c r="I48" s="30">
         <f>IF(D48="","",D48)</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="26" t="n"/>
-      <c r="B49" s="14" t="n"/>
-      <c r="C49" s="14" t="n"/>
-      <c r="D49" s="27" t="n"/>
-      <c r="E49" s="14" t="n"/>
-      <c r="F49" s="14" t="n"/>
-      <c r="G49" s="28">
+      <c r="A49" s="27" t="n"/>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="28" t="n"/>
+      <c r="E49" s="15" t="n"/>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="29">
         <f>IF(C49="","",IF(H49="Income",IF(F49="","Split by rule",F49),IF(OR(F49="",F49="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C49,Settings!$B$19:$B$38,0)),""),F49)))</f>
         <v/>
       </c>
-      <c r="H49" s="28">
+      <c r="H49" s="29">
         <f>IF(C49="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C49,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I49" s="29">
+      <c r="I49" s="30">
         <f>IF(D49="","",D49)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Quadro Free: nota di licenza
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quadro/Quadro-Free.xlsx
+++ b/quadro/Quadro-Free.xlsx
@@ -82,7 +82,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +102,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F2328"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEEE4"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,6 +160,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -893,7 +904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1074,9 +1085,22 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24" ht="36" customHeight="1">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>© 2026 Quadro · All rights reserved</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Quadro Free is free for personal use. You may not resell it, or sell or publish modified versions of it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="9611"/>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C7:D7"/>
@@ -1084,6 +1108,7 @@
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C8:D8"/>
@@ -1149,12 +1174,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Budget year</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="14" t="n">
         <v>2026</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -1174,12 +1199,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Month starts on day</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1204,12 +1229,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Your currency</t>
         </is>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="15">
         <f>IFERROR(INDEX($O$4:$O$29,MATCH('Start Here'!$C$5,$N$4:$N$29,0)),"EUR")</f>
         <v/>
       </c>
@@ -1235,12 +1260,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Month to track (1-12)</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>1</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -1299,17 +1324,17 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Share of income</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Starting balance</t>
         </is>
@@ -1331,15 +1356,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="18" t="n">
         <v>0.55</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1347,7 +1372,7 @@
           <t>55-20-15-10 is the split I recommend, not a must: set the percentages that fit your life.</t>
         </is>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="20">
         <f>B11</f>
         <v/>
       </c>
@@ -1368,15 +1393,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1384,7 +1409,7 @@
           <t>You can also rename the buckets. Only rule: the shares add up to 100%.</t>
         </is>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="20">
         <f>B12</f>
         <v/>
       </c>
@@ -1405,15 +1430,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="18" t="n">
         <v>0.15</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1421,7 +1446,7 @@
           <t>Tip: give each bucket its own pocket or account at your bank (see Start Here).</t>
         </is>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="20">
         <f>B13</f>
         <v/>
       </c>
@@ -1442,18 +1467,18 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="20">
         <f>B14</f>
         <v/>
       </c>
@@ -1474,16 +1499,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="21">
         <f>SUM(C11:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="22">
         <f>IF(ROUND(C15,4)=1,"✓ Adds up to 100%","⚠ Must add up to 100%")</f>
         <v/>
       </c>
@@ -1548,17 +1573,17 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>Default bucket</t>
         </is>
@@ -1575,35 +1600,35 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Salary</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D19" s="15" t="n"/>
+      <c r="D19" s="17" t="n"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Income: money in · Expense: spending · Saving: money set aside (counts against its bucket, not as spending)</t>
         </is>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="20">
         <f>IF(B19="","",COUNTIF($B$19:B19,"?*"))</f>
         <v/>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(1,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(1,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="20">
         <f>IF(OR(B19="",C19="Income"),"",SUMPRODUCT(($B$19:B19&lt;&gt;"")*($C$19:C19&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1619,30 +1644,30 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Extra Income</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D20" s="15" t="n"/>
-      <c r="H20" s="18">
+      <c r="D20" s="17" t="n"/>
+      <c r="H20" s="20">
         <f>IF(B20="","",COUNTIF($B$19:B20,"?*"))</f>
         <v/>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(2,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(2,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L20" s="18">
+      <c r="L20" s="20">
         <f>IF(OR(B20="",C20="Income"),"",SUMPRODUCT(($B$19:B20&lt;&gt;"")*($C$19:C20&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1658,34 +1683,34 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Fixed Costs</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="20">
         <f>IF(B21="","",COUNTIF($B$19:B21,"?*"))</f>
         <v/>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(3,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J21" s="18">
+      <c r="J21" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(3,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L21" s="18">
+      <c r="L21" s="20">
         <f>IF(OR(B21="",C21="Income"),"",SUMPRODUCT(($B$19:B21&lt;&gt;"")*($C$19:C21&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1701,34 +1726,34 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Groceries</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="20">
         <f>IF(B22="","",COUNTIF($B$19:B22,"?*"))</f>
         <v/>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(4,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J22" s="18">
+      <c r="J22" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(4,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L22" s="18">
+      <c r="L22" s="20">
         <f>IF(OR(B22="",C22="Income"),"",SUMPRODUCT(($B$19:B22&lt;&gt;"")*($C$19:C22&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1744,34 +1769,34 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="20">
         <f>IF(B23="","",COUNTIF($B$19:B23,"?*"))</f>
         <v/>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(5,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(5,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L23" s="18">
+      <c r="L23" s="20">
         <f>IF(OR(B23="",C23="Income"),"",SUMPRODUCT(($B$19:B23&lt;&gt;"")*($C$19:C23&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1787,34 +1812,34 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="20">
         <f>IF(B24="","",COUNTIF($B$19:B24,"?*"))</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(6,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="J24" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(6,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L24" s="18">
+      <c r="L24" s="20">
         <f>IF(OR(B24="",C24="Income"),"",SUMPRODUCT(($B$19:B24&lt;&gt;"")*($C$19:C24&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1830,34 +1855,34 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Eating Out</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H25" s="18">
+      <c r="H25" s="20">
         <f>IF(B25="","",COUNTIF($B$19:B25,"?*"))</f>
         <v/>
       </c>
-      <c r="I25" s="18">
+      <c r="I25" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(7,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J25" s="18">
+      <c r="J25" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(7,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L25" s="18">
+      <c r="L25" s="20">
         <f>IF(OR(B25="",C25="Income"),"",SUMPRODUCT(($B$19:B25&lt;&gt;"")*($C$19:C25&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1873,34 +1898,34 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Fun &amp; Shopping</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H26" s="18">
+      <c r="H26" s="20">
         <f>IF(B26="","",COUNTIF($B$19:B26,"?*"))</f>
         <v/>
       </c>
-      <c r="I26" s="18">
+      <c r="I26" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(8,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(8,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L26" s="18">
+      <c r="L26" s="20">
         <f>IF(OR(B26="",C26="Income"),"",SUMPRODUCT(($B$19:B26&lt;&gt;"")*($C$19:C26&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1916,34 +1941,34 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>Gifts</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>Quality of Life</t>
         </is>
       </c>
-      <c r="H27" s="18">
+      <c r="H27" s="20">
         <f>IF(B27="","",COUNTIF($B$19:B27,"?*"))</f>
         <v/>
       </c>
-      <c r="I27" s="18">
+      <c r="I27" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(9,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J27" s="18">
+      <c r="J27" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(9,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L27" s="18">
+      <c r="L27" s="20">
         <f>IF(OR(B27="",C27="Income"),"",SUMPRODUCT(($B$19:B27&lt;&gt;"")*($C$19:C27&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -1959,34 +1984,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="H28" s="18">
+      <c r="H28" s="20">
         <f>IF(B28="","",COUNTIF($B$19:B28,"?*"))</f>
         <v/>
       </c>
-      <c r="I28" s="18">
+      <c r="I28" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(10,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J28" s="18">
+      <c r="J28" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(10,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L28" s="18">
+      <c r="L28" s="20">
         <f>IF(OR(B28="",C28="Income"),"",SUMPRODUCT(($B$19:B28&lt;&gt;"")*($C$19:C28&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -2002,34 +2027,34 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>Saving</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>Safety Fund</t>
         </is>
       </c>
-      <c r="H29" s="18">
+      <c r="H29" s="20">
         <f>IF(B29="","",COUNTIF($B$19:B29,"?*"))</f>
         <v/>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(11,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(11,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L29" s="18">
+      <c r="L29" s="20">
         <f>IF(OR(B29="",C29="Income"),"",SUMPRODUCT(($B$19:B29&lt;&gt;"")*($C$19:C29&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -2045,202 +2070,202 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>Saving</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="H30" s="18">
+      <c r="H30" s="20">
         <f>IF(B30="","",COUNTIF($B$19:B30,"?*"))</f>
         <v/>
       </c>
-      <c r="I30" s="18">
+      <c r="I30" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(12,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J30" s="18">
+      <c r="J30" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(12,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L30" s="18">
+      <c r="L30" s="20">
         <f>IF(OR(B30="",C30="Income"),"",SUMPRODUCT(($B$19:B30&lt;&gt;"")*($C$19:C30&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="H31" s="18">
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="17" t="n"/>
+      <c r="D31" s="17" t="n"/>
+      <c r="H31" s="20">
         <f>IF(B31="","",COUNTIF($B$19:B31,"?*"))</f>
         <v/>
       </c>
-      <c r="I31" s="18">
+      <c r="I31" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(13,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J31" s="18">
+      <c r="J31" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(13,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L31" s="18">
+      <c r="L31" s="20">
         <f>IF(OR(B31="",C31="Income"),"",SUMPRODUCT(($B$19:B31&lt;&gt;"")*($C$19:C31&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="H32" s="18">
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="17" t="n"/>
+      <c r="H32" s="20">
         <f>IF(B32="","",COUNTIF($B$19:B32,"?*"))</f>
         <v/>
       </c>
-      <c r="I32" s="18">
+      <c r="I32" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(14,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J32" s="18">
+      <c r="J32" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(14,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L32" s="18">
+      <c r="L32" s="20">
         <f>IF(OR(B32="",C32="Income"),"",SUMPRODUCT(($B$19:B32&lt;&gt;"")*($C$19:C32&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="H33" s="18">
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="H33" s="20">
         <f>IF(B33="","",COUNTIF($B$19:B33,"?*"))</f>
         <v/>
       </c>
-      <c r="I33" s="18">
+      <c r="I33" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(15,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J33" s="18">
+      <c r="J33" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(15,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L33" s="18">
+      <c r="L33" s="20">
         <f>IF(OR(B33="",C33="Income"),"",SUMPRODUCT(($B$19:B33&lt;&gt;"")*($C$19:C33&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="H34" s="18">
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17" t="n"/>
+      <c r="D34" s="17" t="n"/>
+      <c r="H34" s="20">
         <f>IF(B34="","",COUNTIF($B$19:B34,"?*"))</f>
         <v/>
       </c>
-      <c r="I34" s="18">
+      <c r="I34" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(16,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J34" s="18">
+      <c r="J34" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(16,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L34" s="18">
+      <c r="L34" s="20">
         <f>IF(OR(B34="",C34="Income"),"",SUMPRODUCT(($B$19:B34&lt;&gt;"")*($C$19:C34&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="H35" s="18">
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="17" t="n"/>
+      <c r="D35" s="17" t="n"/>
+      <c r="H35" s="20">
         <f>IF(B35="","",COUNTIF($B$19:B35,"?*"))</f>
         <v/>
       </c>
-      <c r="I35" s="18">
+      <c r="I35" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(17,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J35" s="18">
+      <c r="J35" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(17,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L35" s="18">
+      <c r="L35" s="20">
         <f>IF(OR(B35="",C35="Income"),"",SUMPRODUCT(($B$19:B35&lt;&gt;"")*($C$19:C35&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="H36" s="18">
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="H36" s="20">
         <f>IF(B36="","",COUNTIF($B$19:B36,"?*"))</f>
         <v/>
       </c>
-      <c r="I36" s="18">
+      <c r="I36" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(18,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J36" s="18">
+      <c r="J36" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(18,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L36" s="18">
+      <c r="L36" s="20">
         <f>IF(OR(B36="",C36="Income"),"",SUMPRODUCT(($B$19:B36&lt;&gt;"")*($C$19:C36&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="H37" s="18">
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="17" t="n"/>
+      <c r="D37" s="17" t="n"/>
+      <c r="H37" s="20">
         <f>IF(B37="","",COUNTIF($B$19:B37,"?*"))</f>
         <v/>
       </c>
-      <c r="I37" s="18">
+      <c r="I37" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(19,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J37" s="18">
+      <c r="J37" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(19,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L37" s="18">
+      <c r="L37" s="20">
         <f>IF(OR(B37="",C37="Income"),"",SUMPRODUCT(($B$19:B37&lt;&gt;"")*($C$19:C37&lt;&gt;"Income")))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="H38" s="18">
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="H38" s="20">
         <f>IF(B38="","",COUNTIF($B$19:B38,"?*"))</f>
         <v/>
       </c>
-      <c r="I38" s="18">
+      <c r="I38" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(20,$H$19:$H$38,0)),"")</f>
         <v/>
       </c>
-      <c r="J38" s="18">
+      <c r="J38" s="20">
         <f>IFERROR(INDEX($B$19:$B$38,MATCH(20,$L$19:$L$38,0)),"")</f>
         <v/>
       </c>
-      <c r="L38" s="18">
+      <c r="L38" s="20">
         <f>IF(OR(B38="",C38="Income"),"",SUMPRODUCT(($B$19:B38&lt;&gt;"")*($C$19:C38&lt;&gt;"Income")))</f>
         <v/>
       </c>
@@ -2354,11 +2379,11 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21">
+      <c r="A1" s="23">
         <f>INDEX({"January","February","March","April","May","June","July","August","September","October","November","December"},Settings!$C$7)</f>
         <v/>
       </c>
-      <c r="C1" s="22">
+      <c r="C1" s="24">
         <f>Settings!$C$4</f>
         <v/>
       </c>
@@ -2372,7 +2397,7 @@
           <t>Checks</t>
         </is>
       </c>
-      <c r="ZZ1" s="18">
+      <c r="ZZ1" s="20">
         <f>Settings!$C$6</f>
         <v/>
       </c>
@@ -2383,20 +2408,20 @@
           <t>Period</t>
         </is>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="25">
         <f>DATE(Settings!$C$4,Settings!$C$7-IF(Settings!$C$5=1,0,1),Settings!$C$5)</f>
         <v/>
       </c>
-      <c r="C2" s="23">
+      <c r="C2" s="25">
         <f>DATE(Settings!$C$4,Settings!$C$7+1-IF(Settings!$C$5=1,0,1),Settings!$C$5)-1</f>
         <v/>
       </c>
-      <c r="K2" s="11" t="inlineStr">
+      <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="L2" s="24">
+      <c r="L2" s="26">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income")</f>
         <v/>
       </c>
@@ -2405,18 +2430,18 @@
           <t>Missing category</t>
         </is>
       </c>
-      <c r="P2" s="25">
+      <c r="P2" s="27">
         <f>SUMPRODUCT(($D$10:$D$49&lt;&gt;"")*($C$10:$C$49=""))</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="L3" s="24">
+      <c r="L3" s="26">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Expense")</f>
         <v/>
       </c>
@@ -2425,7 +2450,7 @@
           <t>Unknown category</t>
         </is>
       </c>
-      <c r="P3" s="25">
+      <c r="P3" s="27">
         <f>COUNTIF($H$10:$H$49,"Unknown")</f>
         <v/>
       </c>
@@ -2436,12 +2461,12 @@
           <t>How to use</t>
         </is>
       </c>
-      <c r="K4" s="11" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>Saved &amp; invested</t>
         </is>
       </c>
-      <c r="L4" s="24">
+      <c r="L4" s="26">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Saving")</f>
         <v/>
       </c>
@@ -2450,7 +2475,7 @@
           <t>Dates typed as text</t>
         </is>
       </c>
-      <c r="P4" s="25">
+      <c r="P4" s="27">
         <f>SUMPRODUCT(($A$10:$A$49&lt;&gt;"")*NOT(ISNUMBER($A$10:$A$49)))</f>
         <v/>
       </c>
@@ -2461,12 +2486,12 @@
           <t>Add one row per transaction in the yellow cells. Pick a category: bucket and type fill in by themselves.</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>Left over</t>
         </is>
       </c>
-      <c r="L5" s="24">
+      <c r="L5" s="26">
         <f>L2-L3-L4</f>
         <v/>
       </c>
@@ -2475,7 +2500,7 @@
           <t>Dates outside this period</t>
         </is>
       </c>
-      <c r="P5" s="25">
+      <c r="P5" s="27">
         <f>SUMPRODUCT(ISNUMBER($A$10:$A$49)*((($A$10:$A$49&lt;$B$2)+($A$10:$A$49&gt;$C$2))&gt;0))</f>
         <v/>
       </c>
@@ -2486,7 +2511,7 @@
           <t>Paid with money from another bucket? Choose it in “Paid from / Allocate to”. For income, pick a bucket to put it all there, or leave blank to split it by your rule.</t>
         </is>
       </c>
-      <c r="N6" s="20">
+      <c r="N6" s="22">
         <f>IF(SUM(P2:P5)=0,"✓ All good","⚠ Fix the rows highlighted in red")</f>
         <v/>
       </c>
@@ -2500,358 +2525,358 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="28">
         <f>"Amount"</f>
         <v/>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Paid from / Allocate to</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="I9" s="26">
+      <c r="I9" s="28">
         <f>"In your currency "&amp;"("&amp;Settings!$C$6&amp;")"</f>
         <v/>
       </c>
-      <c r="K9" s="14" t="inlineStr">
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="L9" s="14" t="inlineStr">
+      <c r="L9" s="16" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>
       </c>
-      <c r="M9" s="14" t="inlineStr">
+      <c r="M9" s="16" t="inlineStr">
         <is>
           <t>Carried over</t>
         </is>
       </c>
-      <c r="N9" s="14" t="inlineStr">
+      <c r="N9" s="16" t="inlineStr">
         <is>
           <t>From income</t>
         </is>
       </c>
-      <c r="O9" s="14" t="inlineStr">
+      <c r="O9" s="16" t="inlineStr">
         <is>
           <t>Spent</t>
         </is>
       </c>
-      <c r="P9" s="14" t="inlineStr">
+      <c r="P9" s="16" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
       </c>
-      <c r="Q9" s="14" t="inlineStr">
+      <c r="Q9" s="16" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="n"/>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="29">
+      <c r="A10" s="29" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="31">
         <f>IF(C10="","",IF(H10="Income",IF(F10="","Split by rule",F10),IF(OR(F10="",F10="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C10,Settings!$B$19:$B$38,0)),""),F10)))</f>
         <v/>
       </c>
-      <c r="H10" s="29">
+      <c r="H10" s="31">
         <f>IF(C10="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C10,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="32">
         <f>IF(D10="","",D10)</f>
         <v/>
       </c>
-      <c r="K10" s="31">
+      <c r="K10" s="33">
         <f>Settings!$B$11</f>
         <v/>
       </c>
-      <c r="L10" s="32">
+      <c r="L10" s="34">
         <f>Settings!$C$11</f>
         <v/>
       </c>
-      <c r="M10" s="33">
+      <c r="M10" s="35">
         <f>Settings!$D$11</f>
         <v/>
       </c>
-      <c r="N10" s="33">
+      <c r="N10" s="35">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L10+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K10)</f>
         <v/>
       </c>
-      <c r="O10" s="33">
+      <c r="O10" s="35">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K10,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P10" s="34">
+      <c r="P10" s="36">
         <f>M10+N10-O10</f>
         <v/>
       </c>
-      <c r="Q10" s="33">
+      <c r="Q10" s="35">
         <f>M10+N10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="n"/>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="29">
+      <c r="A11" s="29" t="n"/>
+      <c r="B11" s="17" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="31">
         <f>IF(C11="","",IF(H11="Income",IF(F11="","Split by rule",F11),IF(OR(F11="",F11="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C11,Settings!$B$19:$B$38,0)),""),F11)))</f>
         <v/>
       </c>
-      <c r="H11" s="29">
+      <c r="H11" s="31">
         <f>IF(C11="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C11,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="32">
         <f>IF(D11="","",D11)</f>
         <v/>
       </c>
-      <c r="K11" s="31">
+      <c r="K11" s="33">
         <f>Settings!$B$12</f>
         <v/>
       </c>
-      <c r="L11" s="32">
+      <c r="L11" s="34">
         <f>Settings!$C$12</f>
         <v/>
       </c>
-      <c r="M11" s="33">
+      <c r="M11" s="35">
         <f>Settings!$D$12</f>
         <v/>
       </c>
-      <c r="N11" s="33">
+      <c r="N11" s="35">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L11+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K11)</f>
         <v/>
       </c>
-      <c r="O11" s="33">
+      <c r="O11" s="35">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K11,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="36">
         <f>M11+N11-O11</f>
         <v/>
       </c>
-      <c r="Q11" s="33">
+      <c r="Q11" s="35">
         <f>M11+N11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="n"/>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="29">
+      <c r="A12" s="29" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="31">
         <f>IF(C12="","",IF(H12="Income",IF(F12="","Split by rule",F12),IF(OR(F12="",F12="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C12,Settings!$B$19:$B$38,0)),""),F12)))</f>
         <v/>
       </c>
-      <c r="H12" s="29">
+      <c r="H12" s="31">
         <f>IF(C12="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C12,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="32">
         <f>IF(D12="","",D12)</f>
         <v/>
       </c>
-      <c r="K12" s="31">
+      <c r="K12" s="33">
         <f>Settings!$B$13</f>
         <v/>
       </c>
-      <c r="L12" s="32">
+      <c r="L12" s="34">
         <f>Settings!$C$13</f>
         <v/>
       </c>
-      <c r="M12" s="33">
+      <c r="M12" s="35">
         <f>Settings!$D$13</f>
         <v/>
       </c>
-      <c r="N12" s="33">
+      <c r="N12" s="35">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L12+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K12)</f>
         <v/>
       </c>
-      <c r="O12" s="33">
+      <c r="O12" s="35">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K12,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P12" s="34">
+      <c r="P12" s="36">
         <f>M12+N12-O12</f>
         <v/>
       </c>
-      <c r="Q12" s="33">
+      <c r="Q12" s="35">
         <f>M12+N12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="n"/>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="29">
+      <c r="A13" s="29" t="n"/>
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="30" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="31">
         <f>IF(C13="","",IF(H13="Income",IF(F13="","Split by rule",F13),IF(OR(F13="",F13="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C13,Settings!$B$19:$B$38,0)),""),F13)))</f>
         <v/>
       </c>
-      <c r="H13" s="29">
+      <c r="H13" s="31">
         <f>IF(C13="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C13,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="32">
         <f>IF(D13="","",D13)</f>
         <v/>
       </c>
-      <c r="K13" s="31">
+      <c r="K13" s="33">
         <f>Settings!$B$14</f>
         <v/>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="34">
         <f>Settings!$C$14</f>
         <v/>
       </c>
-      <c r="M13" s="33">
+      <c r="M13" s="35">
         <f>Settings!$D$14</f>
         <v/>
       </c>
-      <c r="N13" s="33">
+      <c r="N13" s="35">
         <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L13+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K13)</f>
         <v/>
       </c>
-      <c r="O13" s="33">
+      <c r="O13" s="35">
         <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K13,$H$10:$H$49,"&lt;&gt;Income")</f>
         <v/>
       </c>
-      <c r="P13" s="34">
+      <c r="P13" s="36">
         <f>M13+N13-O13</f>
         <v/>
       </c>
-      <c r="Q13" s="33">
+      <c r="Q13" s="35">
         <f>M13+N13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="n"/>
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="29">
+      <c r="A14" s="29" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="30" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="31">
         <f>IF(C14="","",IF(H14="Income",IF(F14="","Split by rule",F14),IF(OR(F14="",F14="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C14,Settings!$B$19:$B$38,0)),""),F14)))</f>
         <v/>
       </c>
-      <c r="H14" s="29">
+      <c r="H14" s="31">
         <f>IF(C14="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C14,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="32">
         <f>IF(D14="","",D14)</f>
         <v/>
       </c>
-      <c r="K14" s="11" t="inlineStr">
+      <c r="K14" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="M14" s="24">
+      <c r="M14" s="26">
         <f>SUM(M10:M13)</f>
         <v/>
       </c>
-      <c r="N14" s="24">
+      <c r="N14" s="26">
         <f>SUM(N10:N13)</f>
         <v/>
       </c>
-      <c r="O14" s="24">
+      <c r="O14" s="26">
         <f>SUM(O10:O13)</f>
         <v/>
       </c>
-      <c r="P14" s="24">
+      <c r="P14" s="26">
         <f>SUM(P10:P13)</f>
         <v/>
       </c>
-      <c r="Q14" s="24">
+      <c r="Q14" s="26">
         <f>SUM(Q10:Q13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="n"/>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="28" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="29">
+      <c r="A15" s="29" t="n"/>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="31">
         <f>IF(C15="","",IF(H15="Income",IF(F15="","Split by rule",F15),IF(OR(F15="",F15="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C15,Settings!$B$19:$B$38,0)),""),F15)))</f>
         <v/>
       </c>
-      <c r="H15" s="29">
+      <c r="H15" s="31">
         <f>IF(C15="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C15,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="32">
         <f>IF(D15="","",D15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="n"/>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="28" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="29">
+      <c r="A16" s="29" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="30" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="31">
         <f>IF(C16="","",IF(H16="Income",IF(F16="","Split by rule",F16),IF(OR(F16="",F16="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C16,Settings!$B$19:$B$38,0)),""),F16)))</f>
         <v/>
       </c>
-      <c r="H16" s="29">
+      <c r="H16" s="31">
         <f>IF(C16="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C16,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="32">
         <f>IF(D16="","",D16)</f>
         <v/>
       </c>
@@ -2862,925 +2887,925 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="27" t="n"/>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="28" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="29">
+      <c r="A17" s="29" t="n"/>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="30" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="31">
         <f>IF(C17="","",IF(H17="Income",IF(F17="","Split by rule",F17),IF(OR(F17="",F17="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C17,Settings!$B$19:$B$38,0)),""),F17)))</f>
         <v/>
       </c>
-      <c r="H17" s="29">
+      <c r="H17" s="31">
         <f>IF(C17="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C17,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="32">
         <f>IF(D17="","",D17)</f>
         <v/>
       </c>
-      <c r="K17" s="14" t="inlineStr">
+      <c r="K17" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="L17" s="14" t="inlineStr">
+      <c r="L17" s="16" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="M17" s="14" t="inlineStr">
+      <c r="M17" s="16" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="n"/>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="28" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="29">
+      <c r="A18" s="29" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="31">
         <f>IF(C18="","",IF(H18="Income",IF(F18="","Split by rule",F18),IF(OR(F18="",F18="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C18,Settings!$B$19:$B$38,0)),""),F18)))</f>
         <v/>
       </c>
-      <c r="H18" s="29">
+      <c r="H18" s="31">
         <f>IF(C18="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C18,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I18" s="30">
+      <c r="I18" s="32">
         <f>IF(D18="","",D18)</f>
         <v/>
       </c>
-      <c r="K18" s="35">
+      <c r="K18" s="37">
         <f>Settings!$J$19</f>
         <v/>
       </c>
-      <c r="L18" s="33">
+      <c r="L18" s="35">
         <f>IF(K18="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K18))</f>
         <v/>
       </c>
-      <c r="M18" s="36">
+      <c r="M18" s="38">
         <f>IF(OR(K18="",L38=0),"",L18/L38)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="n"/>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="29">
+      <c r="A19" s="29" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="30" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="31">
         <f>IF(C19="","",IF(H19="Income",IF(F19="","Split by rule",F19),IF(OR(F19="",F19="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C19,Settings!$B$19:$B$38,0)),""),F19)))</f>
         <v/>
       </c>
-      <c r="H19" s="29">
+      <c r="H19" s="31">
         <f>IF(C19="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C19,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I19" s="30">
+      <c r="I19" s="32">
         <f>IF(D19="","",D19)</f>
         <v/>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="37">
         <f>Settings!$J$20</f>
         <v/>
       </c>
-      <c r="L19" s="33">
+      <c r="L19" s="35">
         <f>IF(K19="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K19))</f>
         <v/>
       </c>
-      <c r="M19" s="36">
+      <c r="M19" s="38">
         <f>IF(OR(K19="",L38=0),"",L19/L38)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="n"/>
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="29">
+      <c r="A20" s="29" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="30" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="31">
         <f>IF(C20="","",IF(H20="Income",IF(F20="","Split by rule",F20),IF(OR(F20="",F20="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C20,Settings!$B$19:$B$38,0)),""),F20)))</f>
         <v/>
       </c>
-      <c r="H20" s="29">
+      <c r="H20" s="31">
         <f>IF(C20="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C20,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I20" s="30">
+      <c r="I20" s="32">
         <f>IF(D20="","",D20)</f>
         <v/>
       </c>
-      <c r="K20" s="35">
+      <c r="K20" s="37">
         <f>Settings!$J$21</f>
         <v/>
       </c>
-      <c r="L20" s="33">
+      <c r="L20" s="35">
         <f>IF(K20="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K20))</f>
         <v/>
       </c>
-      <c r="M20" s="36">
+      <c r="M20" s="38">
         <f>IF(OR(K20="",L38=0),"",L20/L38)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="n"/>
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="28" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="29">
+      <c r="A21" s="29" t="n"/>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="30" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="31">
         <f>IF(C21="","",IF(H21="Income",IF(F21="","Split by rule",F21),IF(OR(F21="",F21="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C21,Settings!$B$19:$B$38,0)),""),F21)))</f>
         <v/>
       </c>
-      <c r="H21" s="29">
+      <c r="H21" s="31">
         <f>IF(C21="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C21,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="32">
         <f>IF(D21="","",D21)</f>
         <v/>
       </c>
-      <c r="K21" s="35">
+      <c r="K21" s="37">
         <f>Settings!$J$22</f>
         <v/>
       </c>
-      <c r="L21" s="33">
+      <c r="L21" s="35">
         <f>IF(K21="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K21))</f>
         <v/>
       </c>
-      <c r="M21" s="36">
+      <c r="M21" s="38">
         <f>IF(OR(K21="",L38=0),"",L21/L38)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="n"/>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="28" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="29">
+      <c r="A22" s="29" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="30" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="31">
         <f>IF(C22="","",IF(H22="Income",IF(F22="","Split by rule",F22),IF(OR(F22="",F22="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C22,Settings!$B$19:$B$38,0)),""),F22)))</f>
         <v/>
       </c>
-      <c r="H22" s="29">
+      <c r="H22" s="31">
         <f>IF(C22="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C22,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="32">
         <f>IF(D22="","",D22)</f>
         <v/>
       </c>
-      <c r="K22" s="35">
+      <c r="K22" s="37">
         <f>Settings!$J$23</f>
         <v/>
       </c>
-      <c r="L22" s="33">
+      <c r="L22" s="35">
         <f>IF(K22="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K22))</f>
         <v/>
       </c>
-      <c r="M22" s="36">
+      <c r="M22" s="38">
         <f>IF(OR(K22="",L38=0),"",L22/L38)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="n"/>
-      <c r="B23" s="15" t="n"/>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="15" t="n"/>
-      <c r="F23" s="15" t="n"/>
-      <c r="G23" s="29">
+      <c r="A23" s="29" t="n"/>
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="30" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17" t="n"/>
+      <c r="G23" s="31">
         <f>IF(C23="","",IF(H23="Income",IF(F23="","Split by rule",F23),IF(OR(F23="",F23="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C23,Settings!$B$19:$B$38,0)),""),F23)))</f>
         <v/>
       </c>
-      <c r="H23" s="29">
+      <c r="H23" s="31">
         <f>IF(C23="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C23,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I23" s="30">
+      <c r="I23" s="32">
         <f>IF(D23="","",D23)</f>
         <v/>
       </c>
-      <c r="K23" s="35">
+      <c r="K23" s="37">
         <f>Settings!$J$24</f>
         <v/>
       </c>
-      <c r="L23" s="33">
+      <c r="L23" s="35">
         <f>IF(K23="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K23))</f>
         <v/>
       </c>
-      <c r="M23" s="36">
+      <c r="M23" s="38">
         <f>IF(OR(K23="",L38=0),"",L23/L38)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="28" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="29">
+      <c r="A24" s="29" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="30" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="31">
         <f>IF(C24="","",IF(H24="Income",IF(F24="","Split by rule",F24),IF(OR(F24="",F24="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C24,Settings!$B$19:$B$38,0)),""),F24)))</f>
         <v/>
       </c>
-      <c r="H24" s="29">
+      <c r="H24" s="31">
         <f>IF(C24="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C24,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="32">
         <f>IF(D24="","",D24)</f>
         <v/>
       </c>
-      <c r="K24" s="35">
+      <c r="K24" s="37">
         <f>Settings!$J$25</f>
         <v/>
       </c>
-      <c r="L24" s="33">
+      <c r="L24" s="35">
         <f>IF(K24="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K24))</f>
         <v/>
       </c>
-      <c r="M24" s="36">
+      <c r="M24" s="38">
         <f>IF(OR(K24="",L38=0),"",L24/L38)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="n"/>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="28" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="29">
+      <c r="A25" s="29" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="31">
         <f>IF(C25="","",IF(H25="Income",IF(F25="","Split by rule",F25),IF(OR(F25="",F25="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C25,Settings!$B$19:$B$38,0)),""),F25)))</f>
         <v/>
       </c>
-      <c r="H25" s="29">
+      <c r="H25" s="31">
         <f>IF(C25="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C25,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="32">
         <f>IF(D25="","",D25)</f>
         <v/>
       </c>
-      <c r="K25" s="35">
+      <c r="K25" s="37">
         <f>Settings!$J$26</f>
         <v/>
       </c>
-      <c r="L25" s="33">
+      <c r="L25" s="35">
         <f>IF(K25="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K25))</f>
         <v/>
       </c>
-      <c r="M25" s="36">
+      <c r="M25" s="38">
         <f>IF(OR(K25="",L38=0),"",L25/L38)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="15" t="n"/>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="28" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="29">
+      <c r="A26" s="29" t="n"/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="30" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="31">
         <f>IF(C26="","",IF(H26="Income",IF(F26="","Split by rule",F26),IF(OR(F26="",F26="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C26,Settings!$B$19:$B$38,0)),""),F26)))</f>
         <v/>
       </c>
-      <c r="H26" s="29">
+      <c r="H26" s="31">
         <f>IF(C26="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C26,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I26" s="30">
+      <c r="I26" s="32">
         <f>IF(D26="","",D26)</f>
         <v/>
       </c>
-      <c r="K26" s="35">
+      <c r="K26" s="37">
         <f>Settings!$J$27</f>
         <v/>
       </c>
-      <c r="L26" s="33">
+      <c r="L26" s="35">
         <f>IF(K26="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K26))</f>
         <v/>
       </c>
-      <c r="M26" s="36">
+      <c r="M26" s="38">
         <f>IF(OR(K26="",L38=0),"",L26/L38)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="n"/>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="28" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="29">
+      <c r="A27" s="29" t="n"/>
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="17" t="n"/>
+      <c r="D27" s="30" t="n"/>
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="31">
         <f>IF(C27="","",IF(H27="Income",IF(F27="","Split by rule",F27),IF(OR(F27="",F27="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C27,Settings!$B$19:$B$38,0)),""),F27)))</f>
         <v/>
       </c>
-      <c r="H27" s="29">
+      <c r="H27" s="31">
         <f>IF(C27="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C27,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="32">
         <f>IF(D27="","",D27)</f>
         <v/>
       </c>
-      <c r="K27" s="35">
+      <c r="K27" s="37">
         <f>Settings!$J$28</f>
         <v/>
       </c>
-      <c r="L27" s="33">
+      <c r="L27" s="35">
         <f>IF(K27="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K27))</f>
         <v/>
       </c>
-      <c r="M27" s="36">
+      <c r="M27" s="38">
         <f>IF(OR(K27="",L38=0),"",L27/L38)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="28" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="29">
+      <c r="A28" s="29" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="30" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="31">
         <f>IF(C28="","",IF(H28="Income",IF(F28="","Split by rule",F28),IF(OR(F28="",F28="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C28,Settings!$B$19:$B$38,0)),""),F28)))</f>
         <v/>
       </c>
-      <c r="H28" s="29">
+      <c r="H28" s="31">
         <f>IF(C28="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C28,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I28" s="30">
+      <c r="I28" s="32">
         <f>IF(D28="","",D28)</f>
         <v/>
       </c>
-      <c r="K28" s="35">
+      <c r="K28" s="37">
         <f>Settings!$J$29</f>
         <v/>
       </c>
-      <c r="L28" s="33">
+      <c r="L28" s="35">
         <f>IF(K28="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K28))</f>
         <v/>
       </c>
-      <c r="M28" s="36">
+      <c r="M28" s="38">
         <f>IF(OR(K28="",L38=0),"",L28/L38)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="n"/>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="28" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="29">
+      <c r="A29" s="29" t="n"/>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="30" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="31">
         <f>IF(C29="","",IF(H29="Income",IF(F29="","Split by rule",F29),IF(OR(F29="",F29="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C29,Settings!$B$19:$B$38,0)),""),F29)))</f>
         <v/>
       </c>
-      <c r="H29" s="29">
+      <c r="H29" s="31">
         <f>IF(C29="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C29,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I29" s="30">
+      <c r="I29" s="32">
         <f>IF(D29="","",D29)</f>
         <v/>
       </c>
-      <c r="K29" s="35">
+      <c r="K29" s="37">
         <f>Settings!$J$30</f>
         <v/>
       </c>
-      <c r="L29" s="33">
+      <c r="L29" s="35">
         <f>IF(K29="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K29))</f>
         <v/>
       </c>
-      <c r="M29" s="36">
+      <c r="M29" s="38">
         <f>IF(OR(K29="",L38=0),"",L29/L38)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="n"/>
-      <c r="B30" s="15" t="n"/>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="28" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="29">
+      <c r="A30" s="29" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="30" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="31">
         <f>IF(C30="","",IF(H30="Income",IF(F30="","Split by rule",F30),IF(OR(F30="",F30="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C30,Settings!$B$19:$B$38,0)),""),F30)))</f>
         <v/>
       </c>
-      <c r="H30" s="29">
+      <c r="H30" s="31">
         <f>IF(C30="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C30,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I30" s="30">
+      <c r="I30" s="32">
         <f>IF(D30="","",D30)</f>
         <v/>
       </c>
-      <c r="K30" s="35">
+      <c r="K30" s="37">
         <f>Settings!$J$31</f>
         <v/>
       </c>
-      <c r="L30" s="33">
+      <c r="L30" s="35">
         <f>IF(K30="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K30))</f>
         <v/>
       </c>
-      <c r="M30" s="36">
+      <c r="M30" s="38">
         <f>IF(OR(K30="",L38=0),"",L30/L38)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="n"/>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="28" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="29">
+      <c r="A31" s="29" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="17" t="n"/>
+      <c r="D31" s="30" t="n"/>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="31">
         <f>IF(C31="","",IF(H31="Income",IF(F31="","Split by rule",F31),IF(OR(F31="",F31="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C31,Settings!$B$19:$B$38,0)),""),F31)))</f>
         <v/>
       </c>
-      <c r="H31" s="29">
+      <c r="H31" s="31">
         <f>IF(C31="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C31,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I31" s="30">
+      <c r="I31" s="32">
         <f>IF(D31="","",D31)</f>
         <v/>
       </c>
-      <c r="K31" s="35">
+      <c r="K31" s="37">
         <f>Settings!$J$32</f>
         <v/>
       </c>
-      <c r="L31" s="33">
+      <c r="L31" s="35">
         <f>IF(K31="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K31))</f>
         <v/>
       </c>
-      <c r="M31" s="36">
+      <c r="M31" s="38">
         <f>IF(OR(K31="",L38=0),"",L31/L38)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="29">
+      <c r="A32" s="29" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="30" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="31">
         <f>IF(C32="","",IF(H32="Income",IF(F32="","Split by rule",F32),IF(OR(F32="",F32="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C32,Settings!$B$19:$B$38,0)),""),F32)))</f>
         <v/>
       </c>
-      <c r="H32" s="29">
+      <c r="H32" s="31">
         <f>IF(C32="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C32,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I32" s="30">
+      <c r="I32" s="32">
         <f>IF(D32="","",D32)</f>
         <v/>
       </c>
-      <c r="K32" s="35">
+      <c r="K32" s="37">
         <f>Settings!$J$33</f>
         <v/>
       </c>
-      <c r="L32" s="33">
+      <c r="L32" s="35">
         <f>IF(K32="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K32))</f>
         <v/>
       </c>
-      <c r="M32" s="36">
+      <c r="M32" s="38">
         <f>IF(OR(K32="",L38=0),"",L32/L38)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="28" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="29">
+      <c r="A33" s="29" t="n"/>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="30" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="31">
         <f>IF(C33="","",IF(H33="Income",IF(F33="","Split by rule",F33),IF(OR(F33="",F33="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C33,Settings!$B$19:$B$38,0)),""),F33)))</f>
         <v/>
       </c>
-      <c r="H33" s="29">
+      <c r="H33" s="31">
         <f>IF(C33="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C33,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I33" s="30">
+      <c r="I33" s="32">
         <f>IF(D33="","",D33)</f>
         <v/>
       </c>
-      <c r="K33" s="35">
+      <c r="K33" s="37">
         <f>Settings!$J$34</f>
         <v/>
       </c>
-      <c r="L33" s="33">
+      <c r="L33" s="35">
         <f>IF(K33="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K33))</f>
         <v/>
       </c>
-      <c r="M33" s="36">
+      <c r="M33" s="38">
         <f>IF(OR(K33="",L38=0),"",L33/L38)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="28" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
-      <c r="G34" s="29">
+      <c r="A34" s="29" t="n"/>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17" t="n"/>
+      <c r="D34" s="30" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="31">
         <f>IF(C34="","",IF(H34="Income",IF(F34="","Split by rule",F34),IF(OR(F34="",F34="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C34,Settings!$B$19:$B$38,0)),""),F34)))</f>
         <v/>
       </c>
-      <c r="H34" s="29">
+      <c r="H34" s="31">
         <f>IF(C34="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C34,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I34" s="30">
+      <c r="I34" s="32">
         <f>IF(D34="","",D34)</f>
         <v/>
       </c>
-      <c r="K34" s="35">
+      <c r="K34" s="37">
         <f>Settings!$J$35</f>
         <v/>
       </c>
-      <c r="L34" s="33">
+      <c r="L34" s="35">
         <f>IF(K34="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K34))</f>
         <v/>
       </c>
-      <c r="M34" s="36">
+      <c r="M34" s="38">
         <f>IF(OR(K34="",L38=0),"",L34/L38)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="n"/>
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="28" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15" t="n"/>
-      <c r="G35" s="29">
+      <c r="A35" s="29" t="n"/>
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="17" t="n"/>
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="31">
         <f>IF(C35="","",IF(H35="Income",IF(F35="","Split by rule",F35),IF(OR(F35="",F35="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C35,Settings!$B$19:$B$38,0)),""),F35)))</f>
         <v/>
       </c>
-      <c r="H35" s="29">
+      <c r="H35" s="31">
         <f>IF(C35="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C35,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I35" s="30">
+      <c r="I35" s="32">
         <f>IF(D35="","",D35)</f>
         <v/>
       </c>
-      <c r="K35" s="35">
+      <c r="K35" s="37">
         <f>Settings!$J$36</f>
         <v/>
       </c>
-      <c r="L35" s="33">
+      <c r="L35" s="35">
         <f>IF(K35="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K35))</f>
         <v/>
       </c>
-      <c r="M35" s="36">
+      <c r="M35" s="38">
         <f>IF(OR(K35="",L38=0),"",L35/L38)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15" t="n"/>
-      <c r="G36" s="29">
+      <c r="A36" s="29" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="30" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="31">
         <f>IF(C36="","",IF(H36="Income",IF(F36="","Split by rule",F36),IF(OR(F36="",F36="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C36,Settings!$B$19:$B$38,0)),""),F36)))</f>
         <v/>
       </c>
-      <c r="H36" s="29">
+      <c r="H36" s="31">
         <f>IF(C36="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C36,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I36" s="30">
+      <c r="I36" s="32">
         <f>IF(D36="","",D36)</f>
         <v/>
       </c>
-      <c r="K36" s="35">
+      <c r="K36" s="37">
         <f>Settings!$J$37</f>
         <v/>
       </c>
-      <c r="L36" s="33">
+      <c r="L36" s="35">
         <f>IF(K36="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K36))</f>
         <v/>
       </c>
-      <c r="M36" s="36">
+      <c r="M36" s="38">
         <f>IF(OR(K36="",L38=0),"",L36/L38)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="n"/>
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="28" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15" t="n"/>
-      <c r="G37" s="29">
+      <c r="A37" s="29" t="n"/>
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="17" t="n"/>
+      <c r="D37" s="30" t="n"/>
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="31">
         <f>IF(C37="","",IF(H37="Income",IF(F37="","Split by rule",F37),IF(OR(F37="",F37="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C37,Settings!$B$19:$B$38,0)),""),F37)))</f>
         <v/>
       </c>
-      <c r="H37" s="29">
+      <c r="H37" s="31">
         <f>IF(C37="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C37,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I37" s="30">
+      <c r="I37" s="32">
         <f>IF(D37="","",D37)</f>
         <v/>
       </c>
-      <c r="K37" s="35">
+      <c r="K37" s="37">
         <f>Settings!$J$38</f>
         <v/>
       </c>
-      <c r="L37" s="33">
+      <c r="L37" s="35">
         <f>IF(K37="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K37))</f>
         <v/>
       </c>
-      <c r="M37" s="36">
+      <c r="M37" s="38">
         <f>IF(OR(K37="",L38=0),"",L37/L38)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="n"/>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="28" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="29">
+      <c r="A38" s="29" t="n"/>
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="31">
         <f>IF(C38="","",IF(H38="Income",IF(F38="","Split by rule",F38),IF(OR(F38="",F38="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C38,Settings!$B$19:$B$38,0)),""),F38)))</f>
         <v/>
       </c>
-      <c r="H38" s="29">
+      <c r="H38" s="31">
         <f>IF(C38="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C38,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I38" s="30">
+      <c r="I38" s="32">
         <f>IF(D38="","",D38)</f>
         <v/>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="K38" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="L38" s="24">
+      <c r="L38" s="26">
         <f>SUM(L18:L37)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="28" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15" t="n"/>
-      <c r="G39" s="29">
+      <c r="A39" s="29" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="17" t="n"/>
+      <c r="D39" s="30" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="31">
         <f>IF(C39="","",IF(H39="Income",IF(F39="","Split by rule",F39),IF(OR(F39="",F39="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C39,Settings!$B$19:$B$38,0)),""),F39)))</f>
         <v/>
       </c>
-      <c r="H39" s="29">
+      <c r="H39" s="31">
         <f>IF(C39="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C39,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I39" s="30">
+      <c r="I39" s="32">
         <f>IF(D39="","",D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="n"/>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="28" t="n"/>
-      <c r="E40" s="15" t="n"/>
-      <c r="F40" s="15" t="n"/>
-      <c r="G40" s="29">
+      <c r="A40" s="29" t="n"/>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="17" t="n"/>
+      <c r="D40" s="30" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="31">
         <f>IF(C40="","",IF(H40="Income",IF(F40="","Split by rule",F40),IF(OR(F40="",F40="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C40,Settings!$B$19:$B$38,0)),""),F40)))</f>
         <v/>
       </c>
-      <c r="H40" s="29">
+      <c r="H40" s="31">
         <f>IF(C40="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C40,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I40" s="30">
+      <c r="I40" s="32">
         <f>IF(D40="","",D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="n"/>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="28" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15" t="n"/>
-      <c r="G41" s="29">
+      <c r="A41" s="29" t="n"/>
+      <c r="B41" s="17" t="n"/>
+      <c r="C41" s="17" t="n"/>
+      <c r="D41" s="30" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="17" t="n"/>
+      <c r="G41" s="31">
         <f>IF(C41="","",IF(H41="Income",IF(F41="","Split by rule",F41),IF(OR(F41="",F41="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C41,Settings!$B$19:$B$38,0)),""),F41)))</f>
         <v/>
       </c>
-      <c r="H41" s="29">
+      <c r="H41" s="31">
         <f>IF(C41="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C41,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I41" s="30">
+      <c r="I41" s="32">
         <f>IF(D41="","",D41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="n"/>
-      <c r="B42" s="15" t="n"/>
-      <c r="C42" s="15" t="n"/>
-      <c r="D42" s="28" t="n"/>
-      <c r="E42" s="15" t="n"/>
-      <c r="F42" s="15" t="n"/>
-      <c r="G42" s="29">
+      <c r="A42" s="29" t="n"/>
+      <c r="B42" s="17" t="n"/>
+      <c r="C42" s="17" t="n"/>
+      <c r="D42" s="30" t="n"/>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="31">
         <f>IF(C42="","",IF(H42="Income",IF(F42="","Split by rule",F42),IF(OR(F42="",F42="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C42,Settings!$B$19:$B$38,0)),""),F42)))</f>
         <v/>
       </c>
-      <c r="H42" s="29">
+      <c r="H42" s="31">
         <f>IF(C42="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C42,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I42" s="30">
+      <c r="I42" s="32">
         <f>IF(D42="","",D42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="n"/>
-      <c r="B43" s="15" t="n"/>
-      <c r="C43" s="15" t="n"/>
-      <c r="D43" s="28" t="n"/>
-      <c r="E43" s="15" t="n"/>
-      <c r="F43" s="15" t="n"/>
-      <c r="G43" s="29">
+      <c r="A43" s="29" t="n"/>
+      <c r="B43" s="17" t="n"/>
+      <c r="C43" s="17" t="n"/>
+      <c r="D43" s="30" t="n"/>
+      <c r="E43" s="17" t="n"/>
+      <c r="F43" s="17" t="n"/>
+      <c r="G43" s="31">
         <f>IF(C43="","",IF(H43="Income",IF(F43="","Split by rule",F43),IF(OR(F43="",F43="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C43,Settings!$B$19:$B$38,0)),""),F43)))</f>
         <v/>
       </c>
-      <c r="H43" s="29">
+      <c r="H43" s="31">
         <f>IF(C43="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C43,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I43" s="30">
+      <c r="I43" s="32">
         <f>IF(D43="","",D43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="15" t="n"/>
-      <c r="D44" s="28" t="n"/>
-      <c r="E44" s="15" t="n"/>
-      <c r="F44" s="15" t="n"/>
-      <c r="G44" s="29">
+      <c r="A44" s="29" t="n"/>
+      <c r="B44" s="17" t="n"/>
+      <c r="C44" s="17" t="n"/>
+      <c r="D44" s="30" t="n"/>
+      <c r="E44" s="17" t="n"/>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="31">
         <f>IF(C44="","",IF(H44="Income",IF(F44="","Split by rule",F44),IF(OR(F44="",F44="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C44,Settings!$B$19:$B$38,0)),""),F44)))</f>
         <v/>
       </c>
-      <c r="H44" s="29">
+      <c r="H44" s="31">
         <f>IF(C44="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C44,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I44" s="30">
+      <c r="I44" s="32">
         <f>IF(D44="","",D44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="n"/>
-      <c r="B45" s="15" t="n"/>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="28" t="n"/>
-      <c r="E45" s="15" t="n"/>
-      <c r="F45" s="15" t="n"/>
-      <c r="G45" s="29">
+      <c r="A45" s="29" t="n"/>
+      <c r="B45" s="17" t="n"/>
+      <c r="C45" s="17" t="n"/>
+      <c r="D45" s="30" t="n"/>
+      <c r="E45" s="17" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="31">
         <f>IF(C45="","",IF(H45="Income",IF(F45="","Split by rule",F45),IF(OR(F45="",F45="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C45,Settings!$B$19:$B$38,0)),""),F45)))</f>
         <v/>
       </c>
-      <c r="H45" s="29">
+      <c r="H45" s="31">
         <f>IF(C45="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C45,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I45" s="30">
+      <c r="I45" s="32">
         <f>IF(D45="","",D45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="27" t="n"/>
-      <c r="B46" s="15" t="n"/>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="28" t="n"/>
-      <c r="E46" s="15" t="n"/>
-      <c r="F46" s="15" t="n"/>
-      <c r="G46" s="29">
+      <c r="A46" s="29" t="n"/>
+      <c r="B46" s="17" t="n"/>
+      <c r="C46" s="17" t="n"/>
+      <c r="D46" s="30" t="n"/>
+      <c r="E46" s="17" t="n"/>
+      <c r="F46" s="17" t="n"/>
+      <c r="G46" s="31">
         <f>IF(C46="","",IF(H46="Income",IF(F46="","Split by rule",F46),IF(OR(F46="",F46="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C46,Settings!$B$19:$B$38,0)),""),F46)))</f>
         <v/>
       </c>
-      <c r="H46" s="29">
+      <c r="H46" s="31">
         <f>IF(C46="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C46,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I46" s="30">
+      <c r="I46" s="32">
         <f>IF(D46="","",D46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="27" t="n"/>
-      <c r="B47" s="15" t="n"/>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="28" t="n"/>
-      <c r="E47" s="15" t="n"/>
-      <c r="F47" s="15" t="n"/>
-      <c r="G47" s="29">
+      <c r="A47" s="29" t="n"/>
+      <c r="B47" s="17" t="n"/>
+      <c r="C47" s="17" t="n"/>
+      <c r="D47" s="30" t="n"/>
+      <c r="E47" s="17" t="n"/>
+      <c r="F47" s="17" t="n"/>
+      <c r="G47" s="31">
         <f>IF(C47="","",IF(H47="Income",IF(F47="","Split by rule",F47),IF(OR(F47="",F47="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C47,Settings!$B$19:$B$38,0)),""),F47)))</f>
         <v/>
       </c>
-      <c r="H47" s="29">
+      <c r="H47" s="31">
         <f>IF(C47="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C47,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I47" s="30">
+      <c r="I47" s="32">
         <f>IF(D47="","",D47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="27" t="n"/>
-      <c r="B48" s="15" t="n"/>
-      <c r="C48" s="15" t="n"/>
-      <c r="D48" s="28" t="n"/>
-      <c r="E48" s="15" t="n"/>
-      <c r="F48" s="15" t="n"/>
-      <c r="G48" s="29">
+      <c r="A48" s="29" t="n"/>
+      <c r="B48" s="17" t="n"/>
+      <c r="C48" s="17" t="n"/>
+      <c r="D48" s="30" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="31">
         <f>IF(C48="","",IF(H48="Income",IF(F48="","Split by rule",F48),IF(OR(F48="",F48="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C48,Settings!$B$19:$B$38,0)),""),F48)))</f>
         <v/>
       </c>
-      <c r="H48" s="29">
+      <c r="H48" s="31">
         <f>IF(C48="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C48,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I48" s="30">
+      <c r="I48" s="32">
         <f>IF(D48="","",D48)</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="27" t="n"/>
-      <c r="B49" s="15" t="n"/>
-      <c r="C49" s="15" t="n"/>
-      <c r="D49" s="28" t="n"/>
-      <c r="E49" s="15" t="n"/>
-      <c r="F49" s="15" t="n"/>
-      <c r="G49" s="29">
+      <c r="A49" s="29" t="n"/>
+      <c r="B49" s="17" t="n"/>
+      <c r="C49" s="17" t="n"/>
+      <c r="D49" s="30" t="n"/>
+      <c r="E49" s="17" t="n"/>
+      <c r="F49" s="17" t="n"/>
+      <c r="G49" s="31">
         <f>IF(C49="","",IF(H49="Income",IF(F49="","Split by rule",F49),IF(OR(F49="",F49="Split by rule"),IFERROR(INDEX(Settings!$D$19:$D$38,MATCH(C49,Settings!$B$19:$B$38,0)),""),F49)))</f>
         <v/>
       </c>
-      <c r="H49" s="29">
+      <c r="H49" s="31">
         <f>IF(C49="","",IFERROR(INDEX(Settings!$C$19:$C$38,MATCH(C49,Settings!$B$19:$B$38,0)),"Unknown"))</f>
         <v/>
       </c>
-      <c r="I49" s="30">
+      <c r="I49" s="32">
         <f>IF(D49="","",D49)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Quadro Free: controlli su data e importo mancanti
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/quadro/Quadro-Free.xlsx
+++ b/quadro/Quadro-Free.xlsx
@@ -399,7 +399,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Month'!Q9</f>
+              <f>'Month'!Q12</f>
             </strRef>
           </tx>
           <spPr>
@@ -412,12 +412,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Month'!$K$10:$K$13</f>
+              <f>'Month'!$K$13:$K$16</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Month'!$Q$10:$Q$13</f>
+              <f>'Month'!$Q$13:$Q$16</f>
             </numRef>
           </val>
         </ser>
@@ -426,7 +426,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Month'!O9</f>
+              <f>'Month'!O12</f>
             </strRef>
           </tx>
           <spPr>
@@ -439,12 +439,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Month'!$K$10:$K$13</f>
+              <f>'Month'!$K$13:$K$16</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Month'!$O$10:$O$13</f>
+              <f>'Month'!$O$13:$O$16</f>
             </numRef>
           </val>
         </ser>
@@ -521,12 +521,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Month'!$K$18:$K$29</f>
+              <f>'Month'!$K$21:$K$32</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Month'!$L$18:$L$29</f>
+              <f>'Month'!$L$21:$L$32</f>
             </numRef>
           </val>
         </ser>
@@ -594,7 +594,7 @@
     <from>
       <col>18</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="3240000"/>
@@ -946,7 +946,7 @@
       </c>
     </row>
     <row r="6"/>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="52" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
         <is>
           <t>1. Settings</t>
@@ -2427,11 +2427,11 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Missing category</t>
+          <t>Missing date</t>
         </is>
       </c>
       <c r="P2" s="27">
-        <f>SUMPRODUCT(($D$10:$D$49&lt;&gt;"")*($C$10:$C$49=""))</f>
+        <f>SUMPRODUCT(($D$10:$D$49&lt;&gt;"")*($A$10:$A$49=""))</f>
         <v/>
       </c>
     </row>
@@ -2447,11 +2447,11 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Unknown category</t>
+          <t>Missing amount</t>
         </is>
       </c>
       <c r="P3" s="27">
-        <f>COUNTIF($H$10:$H$49,"Unknown")</f>
+        <f>SUMPRODUCT((($A$10:$A$49&lt;&gt;"")+($B$10:$B$49&lt;&gt;"")+($C$10:$C$49&lt;&gt;"")&gt;0)*($D$10:$D$49=""))</f>
         <v/>
       </c>
     </row>
@@ -2472,11 +2472,11 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Dates typed as text</t>
+          <t>Missing category</t>
         </is>
       </c>
       <c r="P4" s="27">
-        <f>SUMPRODUCT(($A$10:$A$49&lt;&gt;"")*NOT(ISNUMBER($A$10:$A$49)))</f>
+        <f>SUMPRODUCT(($D$10:$D$49&lt;&gt;"")*($C$10:$C$49=""))</f>
         <v/>
       </c>
     </row>
@@ -2497,11 +2497,11 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Dates outside this period</t>
+          <t>Unknown category</t>
         </is>
       </c>
       <c r="P5" s="27">
-        <f>SUMPRODUCT(ISNUMBER($A$10:$A$49)*((($A$10:$A$49&lt;$B$2)+($A$10:$A$49&gt;$C$2))&gt;0))</f>
+        <f>COUNTIF($H$10:$H$49,"Unknown")</f>
         <v/>
       </c>
     </row>
@@ -2511,17 +2511,31 @@
           <t>Paid with money from another bucket? Choose it in “Paid from / Allocate to”. For income, pick a bucket to put it all there, or leave blank to split it by your rule.</t>
         </is>
       </c>
-      <c r="N6" s="22">
-        <f>IF(SUM(P2:P5)=0,"✓ All good","⚠ Fix the rows highlighted in red")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Dates typed as text</t>
+        </is>
+      </c>
+      <c r="P6" s="27">
+        <f>SUMPRODUCT(($A$10:$A$49&lt;&gt;"")*NOT(ISNUMBER($A$10:$A$49)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Dates outside this period</t>
+        </is>
+      </c>
+      <c r="P7" s="27">
+        <f>SUMPRODUCT(ISNUMBER($A$10:$A$49)*((($A$10:$A$49&lt;$B$2)+($A$10:$A$49&gt;$C$2))&gt;0))</f>
+        <v/>
+      </c>
+    </row>
     <row r="8">
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Buckets</t>
-        </is>
+      <c r="N8" s="22">
+        <f>IF(SUM(P2:P7)=0,"✓ All good","⚠ Fix the rows highlighted in red")</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -2567,41 +2581,6 @@
       <c r="I9" s="28">
         <f>"In your currency "&amp;"("&amp;Settings!$C$6&amp;")"</f>
         <v/>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
-        <is>
-          <t>Bucket</t>
-        </is>
-      </c>
-      <c r="L9" s="16" t="inlineStr">
-        <is>
-          <t>Rule</t>
-        </is>
-      </c>
-      <c r="M9" s="16" t="inlineStr">
-        <is>
-          <t>Carried over</t>
-        </is>
-      </c>
-      <c r="N9" s="16" t="inlineStr">
-        <is>
-          <t>From income</t>
-        </is>
-      </c>
-      <c r="O9" s="16" t="inlineStr">
-        <is>
-          <t>Spent</t>
-        </is>
-      </c>
-      <c r="P9" s="16" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
-      </c>
-      <c r="Q9" s="16" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
       </c>
     </row>
     <row r="10">
@@ -2623,34 +2602,6 @@
         <f>IF(D10="","",D10)</f>
         <v/>
       </c>
-      <c r="K10" s="33">
-        <f>Settings!$B$11</f>
-        <v/>
-      </c>
-      <c r="L10" s="34">
-        <f>Settings!$C$11</f>
-        <v/>
-      </c>
-      <c r="M10" s="35">
-        <f>Settings!$D$11</f>
-        <v/>
-      </c>
-      <c r="N10" s="35">
-        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L10+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K10)</f>
-        <v/>
-      </c>
-      <c r="O10" s="35">
-        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K10,$H$10:$H$49,"&lt;&gt;Income")</f>
-        <v/>
-      </c>
-      <c r="P10" s="36">
-        <f>M10+N10-O10</f>
-        <v/>
-      </c>
-      <c r="Q10" s="35">
-        <f>M10+N10</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="n"/>
@@ -2671,33 +2622,10 @@
         <f>IF(D11="","",D11)</f>
         <v/>
       </c>
-      <c r="K11" s="33">
-        <f>Settings!$B$12</f>
-        <v/>
-      </c>
-      <c r="L11" s="34">
-        <f>Settings!$C$12</f>
-        <v/>
-      </c>
-      <c r="M11" s="35">
-        <f>Settings!$D$12</f>
-        <v/>
-      </c>
-      <c r="N11" s="35">
-        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L11+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K11)</f>
-        <v/>
-      </c>
-      <c r="O11" s="35">
-        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K11,$H$10:$H$49,"&lt;&gt;Income")</f>
-        <v/>
-      </c>
-      <c r="P11" s="36">
-        <f>M11+N11-O11</f>
-        <v/>
-      </c>
-      <c r="Q11" s="35">
-        <f>M11+N11</f>
-        <v/>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Buckets</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2719,33 +2647,40 @@
         <f>IF(D12="","",D12)</f>
         <v/>
       </c>
-      <c r="K12" s="33">
-        <f>Settings!$B$13</f>
-        <v/>
-      </c>
-      <c r="L12" s="34">
-        <f>Settings!$C$13</f>
-        <v/>
-      </c>
-      <c r="M12" s="35">
-        <f>Settings!$D$13</f>
-        <v/>
-      </c>
-      <c r="N12" s="35">
-        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L12+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K12)</f>
-        <v/>
-      </c>
-      <c r="O12" s="35">
-        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K12,$H$10:$H$49,"&lt;&gt;Income")</f>
-        <v/>
-      </c>
-      <c r="P12" s="36">
-        <f>M12+N12-O12</f>
-        <v/>
-      </c>
-      <c r="Q12" s="35">
-        <f>M12+N12</f>
-        <v/>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Carried over</t>
+        </is>
+      </c>
+      <c r="N12" s="16" t="inlineStr">
+        <is>
+          <t>From income</t>
+        </is>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>Spent</t>
+        </is>
+      </c>
+      <c r="P12" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="Q12" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2768,15 +2703,15 @@
         <v/>
       </c>
       <c r="K13" s="33">
-        <f>Settings!$B$14</f>
+        <f>Settings!$B$11</f>
         <v/>
       </c>
       <c r="L13" s="34">
-        <f>Settings!$C$14</f>
+        <f>Settings!$C$11</f>
         <v/>
       </c>
       <c r="M13" s="35">
-        <f>Settings!$D$14</f>
+        <f>Settings!$D$11</f>
         <v/>
       </c>
       <c r="N13" s="35">
@@ -2815,29 +2750,32 @@
         <f>IF(D14="","",D14)</f>
         <v/>
       </c>
-      <c r="K14" s="13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="M14" s="26">
-        <f>SUM(M10:M13)</f>
-        <v/>
-      </c>
-      <c r="N14" s="26">
-        <f>SUM(N10:N13)</f>
-        <v/>
-      </c>
-      <c r="O14" s="26">
-        <f>SUM(O10:O13)</f>
-        <v/>
-      </c>
-      <c r="P14" s="26">
-        <f>SUM(P10:P13)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="26">
-        <f>SUM(Q10:Q13)</f>
+      <c r="K14" s="33">
+        <f>Settings!$B$12</f>
+        <v/>
+      </c>
+      <c r="L14" s="34">
+        <f>Settings!$C$12</f>
+        <v/>
+      </c>
+      <c r="M14" s="35">
+        <f>Settings!$D$12</f>
+        <v/>
+      </c>
+      <c r="N14" s="35">
+        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L14+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="35">
+        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K14,$H$10:$H$49,"&lt;&gt;Income")</f>
+        <v/>
+      </c>
+      <c r="P14" s="36">
+        <f>M14+N14-O14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="35">
+        <f>M14+N14</f>
         <v/>
       </c>
     </row>
@@ -2860,6 +2798,34 @@
         <f>IF(D15="","",D15)</f>
         <v/>
       </c>
+      <c r="K15" s="33">
+        <f>Settings!$B$13</f>
+        <v/>
+      </c>
+      <c r="L15" s="34">
+        <f>Settings!$C$13</f>
+        <v/>
+      </c>
+      <c r="M15" s="35">
+        <f>Settings!$D$13</f>
+        <v/>
+      </c>
+      <c r="N15" s="35">
+        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L15+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="35">
+        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K15,$H$10:$H$49,"&lt;&gt;Income")</f>
+        <v/>
+      </c>
+      <c r="P15" s="36">
+        <f>M15+N15-O15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="35">
+        <f>M15+N15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="n"/>
@@ -2880,13 +2846,36 @@
         <f>IF(D16="","",D16)</f>
         <v/>
       </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>By category</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+      <c r="K16" s="33">
+        <f>Settings!$B$14</f>
+        <v/>
+      </c>
+      <c r="L16" s="34">
+        <f>Settings!$C$14</f>
+        <v/>
+      </c>
+      <c r="M16" s="35">
+        <f>Settings!$D$14</f>
+        <v/>
+      </c>
+      <c r="N16" s="35">
+        <f>SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,"Split by rule")*L16+SUMIFS($I$10:$I$49,$H$10:$H$49,"Income",$G$10:$G$49,K16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="35">
+        <f>SUMIFS($I$10:$I$49,$G$10:$G$49,K16,$H$10:$H$49,"&lt;&gt;Income")</f>
+        <v/>
+      </c>
+      <c r="P16" s="36">
+        <f>M16+N16-O16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="35">
+        <f>M16+N16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="29" t="n"/>
       <c r="B17" s="17" t="n"/>
       <c r="C17" s="17" t="n"/>
@@ -2905,20 +2894,30 @@
         <f>IF(D17="","",D17)</f>
         <v/>
       </c>
-      <c r="K17" s="16" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="L17" s="16" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="M17" s="16" t="inlineStr">
-        <is>
-          <t>Share</t>
-        </is>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="M17" s="26">
+        <f>SUM(M13:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="26">
+        <f>SUM(N13:N16)</f>
+        <v/>
+      </c>
+      <c r="O17" s="26">
+        <f>SUM(O13:O16)</f>
+        <v/>
+      </c>
+      <c r="P17" s="26">
+        <f>SUM(P13:P16)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="26">
+        <f>SUM(Q13:Q16)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -2940,18 +2939,6 @@
         <f>IF(D18="","",D18)</f>
         <v/>
       </c>
-      <c r="K18" s="37">
-        <f>Settings!$J$19</f>
-        <v/>
-      </c>
-      <c r="L18" s="35">
-        <f>IF(K18="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K18))</f>
-        <v/>
-      </c>
-      <c r="M18" s="38">
-        <f>IF(OR(K18="",L38=0),"",L18/L38)</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="29" t="n"/>
@@ -2972,17 +2959,10 @@
         <f>IF(D19="","",D19)</f>
         <v/>
       </c>
-      <c r="K19" s="37">
-        <f>Settings!$J$20</f>
-        <v/>
-      </c>
-      <c r="L19" s="35">
-        <f>IF(K19="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K19))</f>
-        <v/>
-      </c>
-      <c r="M19" s="38">
-        <f>IF(OR(K19="",L38=0),"",L19/L38)</f>
-        <v/>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>By category</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -3004,17 +2984,20 @@
         <f>IF(D20="","",D20)</f>
         <v/>
       </c>
-      <c r="K20" s="37">
-        <f>Settings!$J$21</f>
-        <v/>
-      </c>
-      <c r="L20" s="35">
-        <f>IF(K20="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K20))</f>
-        <v/>
-      </c>
-      <c r="M20" s="38">
-        <f>IF(OR(K20="",L38=0),"",L20/L38)</f>
-        <v/>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -3037,7 +3020,7 @@
         <v/>
       </c>
       <c r="K21" s="37">
-        <f>Settings!$J$22</f>
+        <f>Settings!$J$19</f>
         <v/>
       </c>
       <c r="L21" s="35">
@@ -3045,7 +3028,7 @@
         <v/>
       </c>
       <c r="M21" s="38">
-        <f>IF(OR(K21="",L38=0),"",L21/L38)</f>
+        <f>IF(OR(K21="",L41=0),"",L21/L41)</f>
         <v/>
       </c>
     </row>
@@ -3069,7 +3052,7 @@
         <v/>
       </c>
       <c r="K22" s="37">
-        <f>Settings!$J$23</f>
+        <f>Settings!$J$20</f>
         <v/>
       </c>
       <c r="L22" s="35">
@@ -3077,7 +3060,7 @@
         <v/>
       </c>
       <c r="M22" s="38">
-        <f>IF(OR(K22="",L38=0),"",L22/L38)</f>
+        <f>IF(OR(K22="",L41=0),"",L22/L41)</f>
         <v/>
       </c>
     </row>
@@ -3101,7 +3084,7 @@
         <v/>
       </c>
       <c r="K23" s="37">
-        <f>Settings!$J$24</f>
+        <f>Settings!$J$21</f>
         <v/>
       </c>
       <c r="L23" s="35">
@@ -3109,7 +3092,7 @@
         <v/>
       </c>
       <c r="M23" s="38">
-        <f>IF(OR(K23="",L38=0),"",L23/L38)</f>
+        <f>IF(OR(K23="",L41=0),"",L23/L41)</f>
         <v/>
       </c>
     </row>
@@ -3133,7 +3116,7 @@
         <v/>
       </c>
       <c r="K24" s="37">
-        <f>Settings!$J$25</f>
+        <f>Settings!$J$22</f>
         <v/>
       </c>
       <c r="L24" s="35">
@@ -3141,7 +3124,7 @@
         <v/>
       </c>
       <c r="M24" s="38">
-        <f>IF(OR(K24="",L38=0),"",L24/L38)</f>
+        <f>IF(OR(K24="",L41=0),"",L24/L41)</f>
         <v/>
       </c>
     </row>
@@ -3165,7 +3148,7 @@
         <v/>
       </c>
       <c r="K25" s="37">
-        <f>Settings!$J$26</f>
+        <f>Settings!$J$23</f>
         <v/>
       </c>
       <c r="L25" s="35">
@@ -3173,7 +3156,7 @@
         <v/>
       </c>
       <c r="M25" s="38">
-        <f>IF(OR(K25="",L38=0),"",L25/L38)</f>
+        <f>IF(OR(K25="",L41=0),"",L25/L41)</f>
         <v/>
       </c>
     </row>
@@ -3197,7 +3180,7 @@
         <v/>
       </c>
       <c r="K26" s="37">
-        <f>Settings!$J$27</f>
+        <f>Settings!$J$24</f>
         <v/>
       </c>
       <c r="L26" s="35">
@@ -3205,7 +3188,7 @@
         <v/>
       </c>
       <c r="M26" s="38">
-        <f>IF(OR(K26="",L38=0),"",L26/L38)</f>
+        <f>IF(OR(K26="",L41=0),"",L26/L41)</f>
         <v/>
       </c>
     </row>
@@ -3229,7 +3212,7 @@
         <v/>
       </c>
       <c r="K27" s="37">
-        <f>Settings!$J$28</f>
+        <f>Settings!$J$25</f>
         <v/>
       </c>
       <c r="L27" s="35">
@@ -3237,7 +3220,7 @@
         <v/>
       </c>
       <c r="M27" s="38">
-        <f>IF(OR(K27="",L38=0),"",L27/L38)</f>
+        <f>IF(OR(K27="",L41=0),"",L27/L41)</f>
         <v/>
       </c>
     </row>
@@ -3261,7 +3244,7 @@
         <v/>
       </c>
       <c r="K28" s="37">
-        <f>Settings!$J$29</f>
+        <f>Settings!$J$26</f>
         <v/>
       </c>
       <c r="L28" s="35">
@@ -3269,7 +3252,7 @@
         <v/>
       </c>
       <c r="M28" s="38">
-        <f>IF(OR(K28="",L38=0),"",L28/L38)</f>
+        <f>IF(OR(K28="",L41=0),"",L28/L41)</f>
         <v/>
       </c>
     </row>
@@ -3293,7 +3276,7 @@
         <v/>
       </c>
       <c r="K29" s="37">
-        <f>Settings!$J$30</f>
+        <f>Settings!$J$27</f>
         <v/>
       </c>
       <c r="L29" s="35">
@@ -3301,7 +3284,7 @@
         <v/>
       </c>
       <c r="M29" s="38">
-        <f>IF(OR(K29="",L38=0),"",L29/L38)</f>
+        <f>IF(OR(K29="",L41=0),"",L29/L41)</f>
         <v/>
       </c>
     </row>
@@ -3325,7 +3308,7 @@
         <v/>
       </c>
       <c r="K30" s="37">
-        <f>Settings!$J$31</f>
+        <f>Settings!$J$28</f>
         <v/>
       </c>
       <c r="L30" s="35">
@@ -3333,7 +3316,7 @@
         <v/>
       </c>
       <c r="M30" s="38">
-        <f>IF(OR(K30="",L38=0),"",L30/L38)</f>
+        <f>IF(OR(K30="",L41=0),"",L30/L41)</f>
         <v/>
       </c>
     </row>
@@ -3357,7 +3340,7 @@
         <v/>
       </c>
       <c r="K31" s="37">
-        <f>Settings!$J$32</f>
+        <f>Settings!$J$29</f>
         <v/>
       </c>
       <c r="L31" s="35">
@@ -3365,7 +3348,7 @@
         <v/>
       </c>
       <c r="M31" s="38">
-        <f>IF(OR(K31="",L38=0),"",L31/L38)</f>
+        <f>IF(OR(K31="",L41=0),"",L31/L41)</f>
         <v/>
       </c>
     </row>
@@ -3389,7 +3372,7 @@
         <v/>
       </c>
       <c r="K32" s="37">
-        <f>Settings!$J$33</f>
+        <f>Settings!$J$30</f>
         <v/>
       </c>
       <c r="L32" s="35">
@@ -3397,7 +3380,7 @@
         <v/>
       </c>
       <c r="M32" s="38">
-        <f>IF(OR(K32="",L38=0),"",L32/L38)</f>
+        <f>IF(OR(K32="",L41=0),"",L32/L41)</f>
         <v/>
       </c>
     </row>
@@ -3421,7 +3404,7 @@
         <v/>
       </c>
       <c r="K33" s="37">
-        <f>Settings!$J$34</f>
+        <f>Settings!$J$31</f>
         <v/>
       </c>
       <c r="L33" s="35">
@@ -3429,7 +3412,7 @@
         <v/>
       </c>
       <c r="M33" s="38">
-        <f>IF(OR(K33="",L38=0),"",L33/L38)</f>
+        <f>IF(OR(K33="",L41=0),"",L33/L41)</f>
         <v/>
       </c>
     </row>
@@ -3453,7 +3436,7 @@
         <v/>
       </c>
       <c r="K34" s="37">
-        <f>Settings!$J$35</f>
+        <f>Settings!$J$32</f>
         <v/>
       </c>
       <c r="L34" s="35">
@@ -3461,7 +3444,7 @@
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>IF(OR(K34="",L38=0),"",L34/L38)</f>
+        <f>IF(OR(K34="",L41=0),"",L34/L41)</f>
         <v/>
       </c>
     </row>
@@ -3485,7 +3468,7 @@
         <v/>
       </c>
       <c r="K35" s="37">
-        <f>Settings!$J$36</f>
+        <f>Settings!$J$33</f>
         <v/>
       </c>
       <c r="L35" s="35">
@@ -3493,7 +3476,7 @@
         <v/>
       </c>
       <c r="M35" s="38">
-        <f>IF(OR(K35="",L38=0),"",L35/L38)</f>
+        <f>IF(OR(K35="",L41=0),"",L35/L41)</f>
         <v/>
       </c>
     </row>
@@ -3517,7 +3500,7 @@
         <v/>
       </c>
       <c r="K36" s="37">
-        <f>Settings!$J$37</f>
+        <f>Settings!$J$34</f>
         <v/>
       </c>
       <c r="L36" s="35">
@@ -3525,7 +3508,7 @@
         <v/>
       </c>
       <c r="M36" s="38">
-        <f>IF(OR(K36="",L38=0),"",L36/L38)</f>
+        <f>IF(OR(K36="",L41=0),"",L36/L41)</f>
         <v/>
       </c>
     </row>
@@ -3549,7 +3532,7 @@
         <v/>
       </c>
       <c r="K37" s="37">
-        <f>Settings!$J$38</f>
+        <f>Settings!$J$35</f>
         <v/>
       </c>
       <c r="L37" s="35">
@@ -3557,7 +3540,7 @@
         <v/>
       </c>
       <c r="M37" s="38">
-        <f>IF(OR(K37="",L38=0),"",L37/L38)</f>
+        <f>IF(OR(K37="",L41=0),"",L37/L41)</f>
         <v/>
       </c>
     </row>
@@ -3580,13 +3563,16 @@
         <f>IF(D38="","",D38)</f>
         <v/>
       </c>
-      <c r="K38" s="13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="L38" s="26">
-        <f>SUM(L18:L37)</f>
+      <c r="K38" s="37">
+        <f>Settings!$J$36</f>
+        <v/>
+      </c>
+      <c r="L38" s="35">
+        <f>IF(K38="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K38))</f>
+        <v/>
+      </c>
+      <c r="M38" s="38">
+        <f>IF(OR(K38="",L41=0),"",L38/L41)</f>
         <v/>
       </c>
     </row>
@@ -3609,6 +3595,18 @@
         <f>IF(D39="","",D39)</f>
         <v/>
       </c>
+      <c r="K39" s="37">
+        <f>Settings!$J$37</f>
+        <v/>
+      </c>
+      <c r="L39" s="35">
+        <f>IF(K39="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K39))</f>
+        <v/>
+      </c>
+      <c r="M39" s="38">
+        <f>IF(OR(K39="",L41=0),"",L39/L41)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="29" t="n"/>
@@ -3629,6 +3627,18 @@
         <f>IF(D40="","",D40)</f>
         <v/>
       </c>
+      <c r="K40" s="37">
+        <f>Settings!$J$38</f>
+        <v/>
+      </c>
+      <c r="L40" s="35">
+        <f>IF(K40="","",SUMIFS($I$10:$I$49,$C$10:$C$49,K40))</f>
+        <v/>
+      </c>
+      <c r="M40" s="38">
+        <f>IF(OR(K40="",L41=0),"",L40/L41)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="29" t="n"/>
@@ -3649,6 +3659,15 @@
         <f>IF(D41="","",D41)</f>
         <v/>
       </c>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="L41" s="26">
+        <f>SUM(L21:L40)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="29" t="n"/>
@@ -3814,7 +3833,7 @@
   <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="9611"/>
   <conditionalFormatting sqref="A10:I49">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>OR(AND($D10&lt;&gt;"",$C10=""),$H10="Unknown",AND($D10&lt;&gt;"",$I10=""),AND($A10&lt;&gt;"",NOT(ISNUMBER($A10))),AND(ISNUMBER($A10),OR($A10&lt;$B$2,$A10&gt;$C$2)))</formula>
+      <formula>OR(AND($D10&lt;&gt;"",$C10=""),$H10="Unknown",AND($D10&lt;&gt;"",$I10=""),AND($D10&lt;&gt;"",$A10=""),AND(ROW()&gt;=10,$D10="",OR($A10&lt;&gt;"",$B10&lt;&gt;"",$C10&lt;&gt;"")),AND($A10&lt;&gt;"",NOT(ISNUMBER($A10))),AND(ISNUMBER($A10),OR($A10&lt;$B$2,$A10&gt;$C$2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2">
@@ -3837,52 +3856,62 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10:P14">
-    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="0">
+  <conditionalFormatting sqref="P6">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:I49 L2:L5 L18:L38 M10:Q14">
-    <cfRule type="expression" priority="7" dxfId="1">
+  <conditionalFormatting sqref="P7">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P13:P17">
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:I49 L2:L5 L21:L41 M13:Q17">
+    <cfRule type="expression" priority="9" dxfId="1">
       <formula>$ZZ$1="EUR"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="2">
+    <cfRule type="expression" priority="10" dxfId="2">
       <formula>$ZZ$1="USD"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="3">
+    <cfRule type="expression" priority="11" dxfId="3">
       <formula>$ZZ$1="GBP"</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="4">
+    <cfRule type="expression" priority="12" dxfId="4">
       <formula>$ZZ$1="CHF"</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="5">
+    <cfRule type="expression" priority="13" dxfId="5">
       <formula>$ZZ$1="CAD"</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="6">
+    <cfRule type="expression" priority="14" dxfId="6">
       <formula>$ZZ$1="AUD"</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" dxfId="7">
+    <cfRule type="expression" priority="15" dxfId="7">
       <formula>$ZZ$1="JPY"</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="8">
+    <cfRule type="expression" priority="16" dxfId="8">
       <formula>$ZZ$1="SEK"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" dxfId="9">
+    <cfRule type="expression" priority="17" dxfId="9">
       <formula>$ZZ$1="NOK"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" dxfId="10">
+    <cfRule type="expression" priority="18" dxfId="10">
       <formula>$ZZ$1="DKK"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" dxfId="11">
+    <cfRule type="expression" priority="19" dxfId="11">
       <formula>$ZZ$1="PLN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" dxfId="12">
+    <cfRule type="expression" priority="20" dxfId="12">
       <formula>$ZZ$1="BRL"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" dxfId="13">
+    <cfRule type="expression" priority="21" dxfId="13">
       <formula>$ZZ$1="MXN"</formula>
     </cfRule>
-    <cfRule type="expression" priority="20" dxfId="14">
+    <cfRule type="expression" priority="22" dxfId="14">
       <formula>$ZZ$1="INR"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>